<commit_message>
Refresh student data workbook
Updated the Adhiparasakthi student records workbook to include the latest data changes. This commit modifies the Excel file used for stored student information.
</commit_message>
<xml_diff>
--- a/files/Adhiparasakthi Students Data 1.xlsx
+++ b/files/Adhiparasakthi Students Data 1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vigne\Google_Backup\Github\sb4c\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74262C99-C121-4B1F-83CC-E6383FB9A842}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10B87436-3423-4997-A84A-4196033CA334}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E3F0EEA9-6BAE-46A1-95E3-E9CE509FC50B}"/>
   </bookViews>
@@ -2571,12 +2571,6 @@
     <t>Edu#244335</t>
   </si>
   <si>
-    <t>EFIBM26268566789@edunetmail.com</t>
-  </si>
-  <si>
-    <t>Edu#721902</t>
-  </si>
-  <si>
     <t>EFIBM26963340792@edunetmail.com</t>
   </si>
   <si>
@@ -2607,12 +2601,6 @@
     <t>Edu#461981</t>
   </si>
   <si>
-    <t>EFIBM26630872231@edunetmail.com</t>
-  </si>
-  <si>
-    <t>Edu#781997</t>
-  </si>
-  <si>
     <t>EFIBM26782374290@edunetmail.com</t>
   </si>
   <si>
@@ -2817,12 +2805,6 @@
     <t>Edu#842997</t>
   </si>
   <si>
-    <t>EFIBM26363139860@edunetmail.com</t>
-  </si>
-  <si>
-    <t>Edu#576105</t>
-  </si>
-  <si>
     <t>EFIBM26671192948@edunetmail.com</t>
   </si>
   <si>
@@ -2877,12 +2859,6 @@
     <t>Edu#466001</t>
   </si>
   <si>
-    <t>EFIBM26399751281@edunetmail.com</t>
-  </si>
-  <si>
-    <t>Edu#789853</t>
-  </si>
-  <si>
     <t>EFIBM26420476671@edunetmail.com</t>
   </si>
   <si>
@@ -2913,12 +2889,6 @@
     <t>Edu#929690</t>
   </si>
   <si>
-    <t>EFIBM26365745181@edunetmail.com</t>
-  </si>
-  <si>
-    <t>Edu#552173</t>
-  </si>
-  <si>
     <t>EFIBM26186546889@edunetmail.com</t>
   </si>
   <si>
@@ -2931,24 +2901,12 @@
     <t>Edu#675000</t>
   </si>
   <si>
-    <t>EFIBM26602786685@edunetmail.com</t>
-  </si>
-  <si>
-    <t>Edu#192643</t>
-  </si>
-  <si>
     <t>EFIBM26547127422@edunetmail.com</t>
   </si>
   <si>
     <t>Edu#161354</t>
   </si>
   <si>
-    <t>EFIBM26656179421@edunetmail.com</t>
-  </si>
-  <si>
-    <t>Edu#351991</t>
-  </si>
-  <si>
     <t>EFIBM26729250746@edunetmail.com</t>
   </si>
   <si>
@@ -3027,12 +2985,6 @@
     <t>Edu#813279</t>
   </si>
   <si>
-    <t>EFIBM26778629465@edunetmail.com</t>
-  </si>
-  <si>
-    <t>Edu#409736</t>
-  </si>
-  <si>
     <t>EFIBM26797604544@edunetmail.com</t>
   </si>
   <si>
@@ -4087,6 +4039,54 @@
   </si>
   <si>
     <t>EduB5#879054</t>
+  </si>
+  <si>
+    <t>EFIBM26B5831478319@edunetmail.com</t>
+  </si>
+  <si>
+    <t>EduB5#724582</t>
+  </si>
+  <si>
+    <t>EFIBM26B5975455986@edunetmail.com</t>
+  </si>
+  <si>
+    <t>EduB5#555057</t>
+  </si>
+  <si>
+    <t>EFIBM26B5641608072@edunetmail.com</t>
+  </si>
+  <si>
+    <t>EduB5#675561</t>
+  </si>
+  <si>
+    <t>EFIBM26B5794832136@edunetmail.com</t>
+  </si>
+  <si>
+    <t>EduB5#953603</t>
+  </si>
+  <si>
+    <t>EFIBM26B5651048524@edunetmail.com</t>
+  </si>
+  <si>
+    <t>EduB5#898232</t>
+  </si>
+  <si>
+    <t>EFIBM26B5328311810@edunetmail.com</t>
+  </si>
+  <si>
+    <t>EduB5#370453</t>
+  </si>
+  <si>
+    <t>EFIBM26B5697829380@edunetmail.com</t>
+  </si>
+  <si>
+    <t>EduB5#865150</t>
+  </si>
+  <si>
+    <t>EFIBM26B5243461614@edunetmail.com</t>
+  </si>
+  <si>
+    <t>EduB5#998024</t>
   </si>
 </sst>
 </file>
@@ -6194,10 +6194,10 @@
         <v>138</v>
       </c>
       <c r="F68" s="12" t="s">
-        <v>1349</v>
+        <v>1333</v>
       </c>
       <c r="G68" s="12" t="s">
-        <v>1350</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="69" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -6561,11 +6561,11 @@
       <c r="E84" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="F84" s="6" t="s">
-        <v>845</v>
-      </c>
-      <c r="G84" s="8" t="s">
-        <v>846</v>
+      <c r="F84" s="12" t="s">
+        <v>1347</v>
+      </c>
+      <c r="G84" s="12" t="s">
+        <v>1348</v>
       </c>
     </row>
     <row r="85" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -6585,10 +6585,10 @@
         <v>138</v>
       </c>
       <c r="F85" s="6" t="s">
-        <v>847</v>
+        <v>845</v>
       </c>
       <c r="G85" s="8" t="s">
-        <v>848</v>
+        <v>846</v>
       </c>
     </row>
     <row r="86" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -6608,10 +6608,10 @@
         <v>138</v>
       </c>
       <c r="F86" s="6" t="s">
-        <v>849</v>
+        <v>847</v>
       </c>
       <c r="G86" s="8" t="s">
-        <v>850</v>
+        <v>848</v>
       </c>
     </row>
     <row r="87" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -6631,10 +6631,10 @@
         <v>138</v>
       </c>
       <c r="F87" s="6" t="s">
-        <v>851</v>
+        <v>849</v>
       </c>
       <c r="G87" s="8" t="s">
-        <v>852</v>
+        <v>850</v>
       </c>
     </row>
     <row r="88" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -6654,10 +6654,10 @@
         <v>138</v>
       </c>
       <c r="F88" s="6" t="s">
-        <v>853</v>
+        <v>851</v>
       </c>
       <c r="G88" s="8" t="s">
-        <v>854</v>
+        <v>852</v>
       </c>
     </row>
     <row r="89" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -6677,10 +6677,10 @@
         <v>138</v>
       </c>
       <c r="F89" s="6" t="s">
-        <v>855</v>
+        <v>853</v>
       </c>
       <c r="G89" s="8" t="s">
-        <v>856</v>
+        <v>854</v>
       </c>
     </row>
     <row r="90" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -6699,11 +6699,11 @@
       <c r="E90" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="F90" s="6" t="s">
-        <v>857</v>
-      </c>
-      <c r="G90" s="8" t="s">
-        <v>858</v>
+      <c r="F90" s="12" t="s">
+        <v>1349</v>
+      </c>
+      <c r="G90" s="12" t="s">
+        <v>1350</v>
       </c>
     </row>
     <row r="91" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -6723,10 +6723,10 @@
         <v>138</v>
       </c>
       <c r="F91" s="6" t="s">
-        <v>859</v>
+        <v>855</v>
       </c>
       <c r="G91" s="8" t="s">
-        <v>860</v>
+        <v>856</v>
       </c>
     </row>
     <row r="92" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -6746,10 +6746,10 @@
         <v>138</v>
       </c>
       <c r="F92" s="6" t="s">
-        <v>861</v>
+        <v>857</v>
       </c>
       <c r="G92" s="8" t="s">
-        <v>862</v>
+        <v>858</v>
       </c>
     </row>
     <row r="93" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -6769,10 +6769,10 @@
         <v>138</v>
       </c>
       <c r="F93" s="6" t="s">
-        <v>863</v>
+        <v>859</v>
       </c>
       <c r="G93" s="8" t="s">
-        <v>864</v>
+        <v>860</v>
       </c>
     </row>
     <row r="94" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -6792,10 +6792,10 @@
         <v>138</v>
       </c>
       <c r="F94" s="6" t="s">
-        <v>865</v>
+        <v>861</v>
       </c>
       <c r="G94" s="8" t="s">
-        <v>866</v>
+        <v>862</v>
       </c>
     </row>
     <row r="95" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -6815,10 +6815,10 @@
         <v>138</v>
       </c>
       <c r="F95" s="6" t="s">
-        <v>867</v>
+        <v>863</v>
       </c>
       <c r="G95" s="8" t="s">
-        <v>868</v>
+        <v>864</v>
       </c>
     </row>
     <row r="96" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -6838,10 +6838,10 @@
         <v>138</v>
       </c>
       <c r="F96" s="6" t="s">
-        <v>869</v>
+        <v>865</v>
       </c>
       <c r="G96" s="8" t="s">
-        <v>870</v>
+        <v>866</v>
       </c>
     </row>
     <row r="97" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -6861,10 +6861,10 @@
         <v>138</v>
       </c>
       <c r="F97" s="6" t="s">
-        <v>871</v>
+        <v>867</v>
       </c>
       <c r="G97" s="8" t="s">
-        <v>872</v>
+        <v>868</v>
       </c>
     </row>
     <row r="98" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -6884,10 +6884,10 @@
         <v>138</v>
       </c>
       <c r="F98" s="6" t="s">
-        <v>873</v>
+        <v>869</v>
       </c>
       <c r="G98" s="8" t="s">
-        <v>874</v>
+        <v>870</v>
       </c>
     </row>
     <row r="99" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -6907,10 +6907,10 @@
         <v>138</v>
       </c>
       <c r="F99" s="6" t="s">
-        <v>875</v>
+        <v>871</v>
       </c>
       <c r="G99" s="8" t="s">
-        <v>876</v>
+        <v>872</v>
       </c>
     </row>
     <row r="100" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -6930,10 +6930,10 @@
         <v>138</v>
       </c>
       <c r="F100" s="6" t="s">
-        <v>877</v>
+        <v>873</v>
       </c>
       <c r="G100" s="8" t="s">
-        <v>878</v>
+        <v>874</v>
       </c>
     </row>
     <row r="101" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -6953,10 +6953,10 @@
         <v>138</v>
       </c>
       <c r="F101" s="6" t="s">
-        <v>879</v>
+        <v>875</v>
       </c>
       <c r="G101" s="8" t="s">
-        <v>880</v>
+        <v>876</v>
       </c>
     </row>
     <row r="102" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -6976,10 +6976,10 @@
         <v>138</v>
       </c>
       <c r="F102" s="6" t="s">
-        <v>881</v>
+        <v>877</v>
       </c>
       <c r="G102" s="8" t="s">
-        <v>882</v>
+        <v>878</v>
       </c>
     </row>
     <row r="103" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -6999,10 +6999,10 @@
         <v>138</v>
       </c>
       <c r="F103" s="6" t="s">
-        <v>883</v>
+        <v>879</v>
       </c>
       <c r="G103" s="8" t="s">
-        <v>884</v>
+        <v>880</v>
       </c>
     </row>
     <row r="104" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7022,10 +7022,10 @@
         <v>138</v>
       </c>
       <c r="F104" s="6" t="s">
-        <v>885</v>
+        <v>881</v>
       </c>
       <c r="G104" s="8" t="s">
-        <v>886</v>
+        <v>882</v>
       </c>
     </row>
     <row r="105" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7045,10 +7045,10 @@
         <v>138</v>
       </c>
       <c r="F105" s="6" t="s">
-        <v>887</v>
+        <v>883</v>
       </c>
       <c r="G105" s="8" t="s">
-        <v>888</v>
+        <v>884</v>
       </c>
     </row>
     <row r="106" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7068,10 +7068,10 @@
         <v>138</v>
       </c>
       <c r="F106" s="6" t="s">
-        <v>889</v>
+        <v>885</v>
       </c>
       <c r="G106" s="8" t="s">
-        <v>890</v>
+        <v>886</v>
       </c>
     </row>
     <row r="107" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7091,10 +7091,10 @@
         <v>138</v>
       </c>
       <c r="F107" s="6" t="s">
-        <v>891</v>
+        <v>887</v>
       </c>
       <c r="G107" s="8" t="s">
-        <v>892</v>
+        <v>888</v>
       </c>
     </row>
     <row r="108" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7114,10 +7114,10 @@
         <v>138</v>
       </c>
       <c r="F108" s="6" t="s">
-        <v>893</v>
+        <v>889</v>
       </c>
       <c r="G108" s="8" t="s">
-        <v>894</v>
+        <v>890</v>
       </c>
     </row>
     <row r="109" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7137,10 +7137,10 @@
         <v>138</v>
       </c>
       <c r="F109" s="6" t="s">
-        <v>895</v>
+        <v>891</v>
       </c>
       <c r="G109" s="8" t="s">
-        <v>896</v>
+        <v>892</v>
       </c>
     </row>
     <row r="110" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7160,10 +7160,10 @@
         <v>138</v>
       </c>
       <c r="F110" s="6" t="s">
-        <v>897</v>
+        <v>893</v>
       </c>
       <c r="G110" s="8" t="s">
-        <v>898</v>
+        <v>894</v>
       </c>
     </row>
     <row r="111" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7183,10 +7183,10 @@
         <v>138</v>
       </c>
       <c r="F111" s="6" t="s">
-        <v>899</v>
+        <v>895</v>
       </c>
       <c r="G111" s="8" t="s">
-        <v>900</v>
+        <v>896</v>
       </c>
     </row>
     <row r="112" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7206,10 +7206,10 @@
         <v>138</v>
       </c>
       <c r="F112" s="6" t="s">
-        <v>901</v>
+        <v>897</v>
       </c>
       <c r="G112" s="8" t="s">
-        <v>902</v>
+        <v>898</v>
       </c>
     </row>
     <row r="113" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7229,10 +7229,10 @@
         <v>138</v>
       </c>
       <c r="F113" s="6" t="s">
-        <v>903</v>
+        <v>899</v>
       </c>
       <c r="G113" s="8" t="s">
-        <v>904</v>
+        <v>900</v>
       </c>
     </row>
     <row r="114" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7252,10 +7252,10 @@
         <v>138</v>
       </c>
       <c r="F114" s="6" t="s">
-        <v>905</v>
+        <v>901</v>
       </c>
       <c r="G114" s="8" t="s">
-        <v>906</v>
+        <v>902</v>
       </c>
     </row>
     <row r="115" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7275,10 +7275,10 @@
         <v>138</v>
       </c>
       <c r="F115" s="6" t="s">
-        <v>907</v>
+        <v>903</v>
       </c>
       <c r="G115" s="8" t="s">
-        <v>908</v>
+        <v>904</v>
       </c>
     </row>
     <row r="116" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7298,10 +7298,10 @@
         <v>138</v>
       </c>
       <c r="F116" s="6" t="s">
-        <v>909</v>
+        <v>905</v>
       </c>
       <c r="G116" s="8" t="s">
-        <v>910</v>
+        <v>906</v>
       </c>
     </row>
     <row r="117" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7321,10 +7321,10 @@
         <v>138</v>
       </c>
       <c r="F117" s="6" t="s">
-        <v>911</v>
+        <v>907</v>
       </c>
       <c r="G117" s="8" t="s">
-        <v>912</v>
+        <v>908</v>
       </c>
     </row>
     <row r="118" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7344,10 +7344,10 @@
         <v>138</v>
       </c>
       <c r="F118" s="6" t="s">
-        <v>913</v>
+        <v>909</v>
       </c>
       <c r="G118" s="8" t="s">
-        <v>914</v>
+        <v>910</v>
       </c>
     </row>
     <row r="119" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7367,10 +7367,10 @@
         <v>138</v>
       </c>
       <c r="F119" s="6" t="s">
-        <v>915</v>
+        <v>911</v>
       </c>
       <c r="G119" s="8" t="s">
-        <v>916</v>
+        <v>912</v>
       </c>
     </row>
     <row r="120" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7390,10 +7390,10 @@
         <v>138</v>
       </c>
       <c r="F120" s="6" t="s">
-        <v>917</v>
+        <v>913</v>
       </c>
       <c r="G120" s="8" t="s">
-        <v>918</v>
+        <v>914</v>
       </c>
     </row>
     <row r="121" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7413,10 +7413,10 @@
         <v>138</v>
       </c>
       <c r="F121" s="6" t="s">
-        <v>919</v>
+        <v>915</v>
       </c>
       <c r="G121" s="8" t="s">
-        <v>920</v>
+        <v>916</v>
       </c>
     </row>
     <row r="122" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7436,10 +7436,10 @@
         <v>138</v>
       </c>
       <c r="F122" s="6" t="s">
-        <v>921</v>
+        <v>917</v>
       </c>
       <c r="G122" s="8" t="s">
-        <v>922</v>
+        <v>918</v>
       </c>
     </row>
     <row r="123" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7459,10 +7459,10 @@
         <v>138</v>
       </c>
       <c r="F123" s="6" t="s">
-        <v>923</v>
+        <v>919</v>
       </c>
       <c r="G123" s="8" t="s">
-        <v>924</v>
+        <v>920</v>
       </c>
     </row>
     <row r="124" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7482,10 +7482,10 @@
         <v>138</v>
       </c>
       <c r="F124" s="6" t="s">
-        <v>925</v>
+        <v>921</v>
       </c>
       <c r="G124" s="8" t="s">
-        <v>926</v>
+        <v>922</v>
       </c>
     </row>
     <row r="125" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7504,11 +7504,11 @@
       <c r="E125" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="F125" s="6" t="s">
-        <v>927</v>
-      </c>
-      <c r="G125" s="8" t="s">
-        <v>928</v>
+      <c r="F125" s="12" t="s">
+        <v>1339</v>
+      </c>
+      <c r="G125" s="12" t="s">
+        <v>1340</v>
       </c>
     </row>
     <row r="126" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7528,10 +7528,10 @@
         <v>138</v>
       </c>
       <c r="F126" s="6" t="s">
-        <v>929</v>
+        <v>923</v>
       </c>
       <c r="G126" s="8" t="s">
-        <v>930</v>
+        <v>924</v>
       </c>
     </row>
     <row r="127" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7551,10 +7551,10 @@
         <v>138</v>
       </c>
       <c r="F127" s="6" t="s">
-        <v>931</v>
+        <v>925</v>
       </c>
       <c r="G127" s="8" t="s">
-        <v>932</v>
+        <v>926</v>
       </c>
     </row>
     <row r="128" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7574,10 +7574,10 @@
         <v>138</v>
       </c>
       <c r="F128" s="6" t="s">
-        <v>933</v>
+        <v>927</v>
       </c>
       <c r="G128" s="8" t="s">
-        <v>934</v>
+        <v>928</v>
       </c>
     </row>
     <row r="129" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7597,10 +7597,10 @@
         <v>138</v>
       </c>
       <c r="F129" s="6" t="s">
-        <v>935</v>
+        <v>929</v>
       </c>
       <c r="G129" s="8" t="s">
-        <v>936</v>
+        <v>930</v>
       </c>
     </row>
     <row r="130" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7620,10 +7620,10 @@
         <v>138</v>
       </c>
       <c r="F130" s="6" t="s">
-        <v>937</v>
+        <v>931</v>
       </c>
       <c r="G130" s="8" t="s">
-        <v>938</v>
+        <v>932</v>
       </c>
     </row>
     <row r="131" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7643,10 +7643,10 @@
         <v>138</v>
       </c>
       <c r="F131" s="6" t="s">
-        <v>939</v>
+        <v>933</v>
       </c>
       <c r="G131" s="8" t="s">
-        <v>940</v>
+        <v>934</v>
       </c>
     </row>
     <row r="132" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7666,10 +7666,10 @@
         <v>138</v>
       </c>
       <c r="F132" s="6" t="s">
-        <v>941</v>
+        <v>935</v>
       </c>
       <c r="G132" s="8" t="s">
-        <v>942</v>
+        <v>936</v>
       </c>
     </row>
     <row r="133" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7689,10 +7689,10 @@
         <v>138</v>
       </c>
       <c r="F133" s="6" t="s">
-        <v>943</v>
+        <v>937</v>
       </c>
       <c r="G133" s="8" t="s">
-        <v>944</v>
+        <v>938</v>
       </c>
     </row>
     <row r="134" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7712,10 +7712,10 @@
         <v>138</v>
       </c>
       <c r="F134" s="6" t="s">
-        <v>945</v>
+        <v>939</v>
       </c>
       <c r="G134" s="8" t="s">
-        <v>946</v>
+        <v>940</v>
       </c>
     </row>
     <row r="135" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7734,11 +7734,11 @@
       <c r="E135" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="F135" s="6" t="s">
-        <v>947</v>
-      </c>
-      <c r="G135" s="8" t="s">
-        <v>948</v>
+      <c r="F135" s="12" t="s">
+        <v>1345</v>
+      </c>
+      <c r="G135" s="12" t="s">
+        <v>1346</v>
       </c>
     </row>
     <row r="136" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7758,10 +7758,10 @@
         <v>138</v>
       </c>
       <c r="F136" s="6" t="s">
-        <v>949</v>
+        <v>941</v>
       </c>
       <c r="G136" s="8" t="s">
-        <v>950</v>
+        <v>942</v>
       </c>
     </row>
     <row r="137" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7781,10 +7781,10 @@
         <v>138</v>
       </c>
       <c r="F137" s="6" t="s">
-        <v>951</v>
+        <v>943</v>
       </c>
       <c r="G137" s="8" t="s">
-        <v>952</v>
+        <v>944</v>
       </c>
     </row>
     <row r="138" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7804,10 +7804,10 @@
         <v>138</v>
       </c>
       <c r="F138" s="6" t="s">
-        <v>953</v>
+        <v>945</v>
       </c>
       <c r="G138" s="8" t="s">
-        <v>954</v>
+        <v>946</v>
       </c>
     </row>
     <row r="139" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7827,10 +7827,10 @@
         <v>138</v>
       </c>
       <c r="F139" s="6" t="s">
-        <v>955</v>
+        <v>947</v>
       </c>
       <c r="G139" s="8" t="s">
-        <v>956</v>
+        <v>948</v>
       </c>
     </row>
     <row r="140" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7850,10 +7850,10 @@
         <v>138</v>
       </c>
       <c r="F140" s="6" t="s">
-        <v>957</v>
+        <v>949</v>
       </c>
       <c r="G140" s="8" t="s">
-        <v>958</v>
+        <v>950</v>
       </c>
     </row>
     <row r="141" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7872,11 +7872,11 @@
       <c r="E141" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="F141" s="6" t="s">
-        <v>959</v>
-      </c>
-      <c r="G141" s="8" t="s">
-        <v>960</v>
+      <c r="F141" s="12" t="s">
+        <v>1335</v>
+      </c>
+      <c r="G141" s="12" t="s">
+        <v>1336</v>
       </c>
     </row>
     <row r="142" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7896,10 +7896,10 @@
         <v>138</v>
       </c>
       <c r="F142" s="6" t="s">
-        <v>961</v>
+        <v>951</v>
       </c>
       <c r="G142" s="8" t="s">
-        <v>962</v>
+        <v>952</v>
       </c>
     </row>
     <row r="143" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7919,10 +7919,10 @@
         <v>138</v>
       </c>
       <c r="F143" s="6" t="s">
-        <v>963</v>
+        <v>953</v>
       </c>
       <c r="G143" s="8" t="s">
-        <v>964</v>
+        <v>954</v>
       </c>
     </row>
     <row r="144" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7941,11 +7941,11 @@
       <c r="E144" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="F144" s="6" t="s">
-        <v>965</v>
-      </c>
-      <c r="G144" s="8" t="s">
-        <v>966</v>
+      <c r="F144" s="12" t="s">
+        <v>1337</v>
+      </c>
+      <c r="G144" s="12" t="s">
+        <v>1338</v>
       </c>
     </row>
     <row r="145" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7965,10 +7965,10 @@
         <v>138</v>
       </c>
       <c r="F145" s="6" t="s">
-        <v>967</v>
+        <v>955</v>
       </c>
       <c r="G145" s="8" t="s">
-        <v>968</v>
+        <v>956</v>
       </c>
     </row>
     <row r="146" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7987,11 +7987,11 @@
       <c r="E146" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="F146" s="6" t="s">
-        <v>969</v>
-      </c>
-      <c r="G146" s="8" t="s">
-        <v>970</v>
+      <c r="F146" s="12" t="s">
+        <v>1343</v>
+      </c>
+      <c r="G146" s="12" t="s">
+        <v>1344</v>
       </c>
     </row>
     <row r="147" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8011,10 +8011,10 @@
         <v>138</v>
       </c>
       <c r="F147" s="6" t="s">
-        <v>971</v>
+        <v>957</v>
       </c>
       <c r="G147" s="8" t="s">
-        <v>972</v>
+        <v>958</v>
       </c>
     </row>
     <row r="148" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8034,10 +8034,10 @@
         <v>138</v>
       </c>
       <c r="F148" s="6" t="s">
-        <v>973</v>
+        <v>959</v>
       </c>
       <c r="G148" s="8" t="s">
-        <v>974</v>
+        <v>960</v>
       </c>
     </row>
     <row r="149" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8057,10 +8057,10 @@
         <v>138</v>
       </c>
       <c r="F149" s="6" t="s">
-        <v>975</v>
+        <v>961</v>
       </c>
       <c r="G149" s="8" t="s">
-        <v>976</v>
+        <v>962</v>
       </c>
     </row>
     <row r="150" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8080,10 +8080,10 @@
         <v>138</v>
       </c>
       <c r="F150" s="6" t="s">
-        <v>977</v>
+        <v>963</v>
       </c>
       <c r="G150" s="8" t="s">
-        <v>978</v>
+        <v>964</v>
       </c>
     </row>
     <row r="151" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8103,10 +8103,10 @@
         <v>138</v>
       </c>
       <c r="F151" s="6" t="s">
-        <v>979</v>
+        <v>965</v>
       </c>
       <c r="G151" s="8" t="s">
-        <v>980</v>
+        <v>966</v>
       </c>
     </row>
     <row r="152" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8126,10 +8126,10 @@
         <v>138</v>
       </c>
       <c r="F152" s="6" t="s">
-        <v>981</v>
+        <v>967</v>
       </c>
       <c r="G152" s="8" t="s">
-        <v>982</v>
+        <v>968</v>
       </c>
     </row>
     <row r="153" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8149,10 +8149,10 @@
         <v>138</v>
       </c>
       <c r="F153" s="6" t="s">
-        <v>983</v>
+        <v>969</v>
       </c>
       <c r="G153" s="8" t="s">
-        <v>984</v>
+        <v>970</v>
       </c>
     </row>
     <row r="154" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8172,10 +8172,10 @@
         <v>138</v>
       </c>
       <c r="F154" s="6" t="s">
-        <v>985</v>
+        <v>971</v>
       </c>
       <c r="G154" s="8" t="s">
-        <v>986</v>
+        <v>972</v>
       </c>
     </row>
     <row r="155" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8195,10 +8195,10 @@
         <v>138</v>
       </c>
       <c r="F155" s="6" t="s">
-        <v>987</v>
+        <v>973</v>
       </c>
       <c r="G155" s="8" t="s">
-        <v>988</v>
+        <v>974</v>
       </c>
     </row>
     <row r="156" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8218,10 +8218,10 @@
         <v>138</v>
       </c>
       <c r="F156" s="6" t="s">
-        <v>989</v>
+        <v>975</v>
       </c>
       <c r="G156" s="8" t="s">
-        <v>990</v>
+        <v>976</v>
       </c>
     </row>
     <row r="157" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8241,10 +8241,10 @@
         <v>138</v>
       </c>
       <c r="F157" s="6" t="s">
-        <v>991</v>
+        <v>977</v>
       </c>
       <c r="G157" s="8" t="s">
-        <v>992</v>
+        <v>978</v>
       </c>
     </row>
     <row r="158" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8264,10 +8264,10 @@
         <v>138</v>
       </c>
       <c r="F158" s="6" t="s">
-        <v>993</v>
+        <v>979</v>
       </c>
       <c r="G158" s="8" t="s">
-        <v>994</v>
+        <v>980</v>
       </c>
     </row>
     <row r="159" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8287,10 +8287,10 @@
         <v>138</v>
       </c>
       <c r="F159" s="6" t="s">
-        <v>995</v>
+        <v>981</v>
       </c>
       <c r="G159" s="8" t="s">
-        <v>996</v>
+        <v>982</v>
       </c>
     </row>
     <row r="160" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8309,11 +8309,11 @@
       <c r="E160" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="F160" s="6" t="s">
-        <v>997</v>
-      </c>
-      <c r="G160" s="8" t="s">
-        <v>998</v>
+      <c r="F160" s="12" t="s">
+        <v>1341</v>
+      </c>
+      <c r="G160" s="12" t="s">
+        <v>1342</v>
       </c>
     </row>
     <row r="161" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8333,10 +8333,10 @@
         <v>138</v>
       </c>
       <c r="F161" s="6" t="s">
-        <v>999</v>
+        <v>983</v>
       </c>
       <c r="G161" s="8" t="s">
-        <v>1000</v>
+        <v>984</v>
       </c>
     </row>
     <row r="162" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8356,10 +8356,10 @@
         <v>138</v>
       </c>
       <c r="F162" s="6" t="s">
-        <v>1001</v>
+        <v>985</v>
       </c>
       <c r="G162" s="8" t="s">
-        <v>1002</v>
+        <v>986</v>
       </c>
     </row>
     <row r="163" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8379,10 +8379,10 @@
         <v>138</v>
       </c>
       <c r="F163" s="6" t="s">
-        <v>1003</v>
+        <v>987</v>
       </c>
       <c r="G163" s="8" t="s">
-        <v>1004</v>
+        <v>988</v>
       </c>
     </row>
     <row r="164" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8402,10 +8402,10 @@
         <v>138</v>
       </c>
       <c r="F164" s="6" t="s">
-        <v>1005</v>
+        <v>989</v>
       </c>
       <c r="G164" s="8" t="s">
-        <v>1006</v>
+        <v>990</v>
       </c>
     </row>
     <row r="165" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8425,10 +8425,10 @@
         <v>138</v>
       </c>
       <c r="F165" s="6" t="s">
-        <v>1007</v>
+        <v>991</v>
       </c>
       <c r="G165" s="8" t="s">
-        <v>1008</v>
+        <v>992</v>
       </c>
     </row>
     <row r="166" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8448,10 +8448,10 @@
         <v>138</v>
       </c>
       <c r="F166" s="6" t="s">
-        <v>1009</v>
+        <v>993</v>
       </c>
       <c r="G166" s="8" t="s">
-        <v>1010</v>
+        <v>994</v>
       </c>
     </row>
     <row r="167" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8471,10 +8471,10 @@
         <v>138</v>
       </c>
       <c r="F167" s="6" t="s">
-        <v>1011</v>
+        <v>995</v>
       </c>
       <c r="G167" s="8" t="s">
-        <v>1012</v>
+        <v>996</v>
       </c>
     </row>
     <row r="168" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8494,10 +8494,10 @@
         <v>138</v>
       </c>
       <c r="F168" s="6" t="s">
-        <v>1013</v>
+        <v>997</v>
       </c>
       <c r="G168" s="8" t="s">
-        <v>1014</v>
+        <v>998</v>
       </c>
     </row>
     <row r="169" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8517,10 +8517,10 @@
         <v>138</v>
       </c>
       <c r="F169" s="6" t="s">
-        <v>1015</v>
+        <v>999</v>
       </c>
       <c r="G169" s="8" t="s">
-        <v>1016</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="170" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8540,10 +8540,10 @@
         <v>138</v>
       </c>
       <c r="F170" s="6" t="s">
-        <v>1017</v>
+        <v>1001</v>
       </c>
       <c r="G170" s="8" t="s">
-        <v>1018</v>
+        <v>1002</v>
       </c>
     </row>
     <row r="171" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8563,10 +8563,10 @@
         <v>138</v>
       </c>
       <c r="F171" s="6" t="s">
-        <v>1019</v>
+        <v>1003</v>
       </c>
       <c r="G171" s="8" t="s">
-        <v>1020</v>
+        <v>1004</v>
       </c>
     </row>
     <row r="172" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8586,10 +8586,10 @@
         <v>138</v>
       </c>
       <c r="F172" s="6" t="s">
-        <v>1021</v>
+        <v>1005</v>
       </c>
       <c r="G172" s="8" t="s">
-        <v>1022</v>
+        <v>1006</v>
       </c>
     </row>
     <row r="173" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8609,10 +8609,10 @@
         <v>138</v>
       </c>
       <c r="F173" s="6" t="s">
-        <v>1023</v>
+        <v>1007</v>
       </c>
       <c r="G173" s="8" t="s">
-        <v>1024</v>
+        <v>1008</v>
       </c>
     </row>
     <row r="174" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8632,10 +8632,10 @@
         <v>138</v>
       </c>
       <c r="F174" s="6" t="s">
-        <v>1025</v>
+        <v>1009</v>
       </c>
       <c r="G174" s="8" t="s">
-        <v>1026</v>
+        <v>1010</v>
       </c>
     </row>
     <row r="175" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8655,10 +8655,10 @@
         <v>138</v>
       </c>
       <c r="F175" s="6" t="s">
-        <v>1027</v>
+        <v>1011</v>
       </c>
       <c r="G175" s="8" t="s">
-        <v>1028</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="176" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8678,10 +8678,10 @@
         <v>138</v>
       </c>
       <c r="F176" s="6" t="s">
-        <v>1029</v>
+        <v>1013</v>
       </c>
       <c r="G176" s="8" t="s">
-        <v>1030</v>
+        <v>1014</v>
       </c>
     </row>
     <row r="177" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8701,10 +8701,10 @@
         <v>138</v>
       </c>
       <c r="F177" s="6" t="s">
-        <v>1031</v>
+        <v>1015</v>
       </c>
       <c r="G177" s="8" t="s">
-        <v>1032</v>
+        <v>1016</v>
       </c>
     </row>
     <row r="178" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8724,10 +8724,10 @@
         <v>138</v>
       </c>
       <c r="F178" s="6" t="s">
-        <v>1033</v>
+        <v>1017</v>
       </c>
       <c r="G178" s="8" t="s">
-        <v>1034</v>
+        <v>1018</v>
       </c>
     </row>
     <row r="179" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8747,10 +8747,10 @@
         <v>138</v>
       </c>
       <c r="F179" s="6" t="s">
-        <v>1035</v>
+        <v>1019</v>
       </c>
       <c r="G179" s="8" t="s">
-        <v>1036</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="180" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8770,10 +8770,10 @@
         <v>138</v>
       </c>
       <c r="F180" s="6" t="s">
-        <v>1037</v>
+        <v>1021</v>
       </c>
       <c r="G180" s="8" t="s">
-        <v>1038</v>
+        <v>1022</v>
       </c>
     </row>
     <row r="181" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8793,10 +8793,10 @@
         <v>138</v>
       </c>
       <c r="F181" s="6" t="s">
-        <v>1039</v>
+        <v>1023</v>
       </c>
       <c r="G181" s="8" t="s">
-        <v>1040</v>
+        <v>1024</v>
       </c>
     </row>
     <row r="182" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8816,10 +8816,10 @@
         <v>138</v>
       </c>
       <c r="F182" s="6" t="s">
-        <v>1041</v>
+        <v>1025</v>
       </c>
       <c r="G182" s="8" t="s">
-        <v>1042</v>
+        <v>1026</v>
       </c>
     </row>
     <row r="183" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8839,10 +8839,10 @@
         <v>138</v>
       </c>
       <c r="F183" s="6" t="s">
-        <v>1043</v>
+        <v>1027</v>
       </c>
       <c r="G183" s="8" t="s">
-        <v>1044</v>
+        <v>1028</v>
       </c>
     </row>
     <row r="184" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8862,10 +8862,10 @@
         <v>138</v>
       </c>
       <c r="F184" s="6" t="s">
-        <v>1045</v>
+        <v>1029</v>
       </c>
       <c r="G184" s="8" t="s">
-        <v>1046</v>
+        <v>1030</v>
       </c>
     </row>
     <row r="185" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8885,10 +8885,10 @@
         <v>138</v>
       </c>
       <c r="F185" s="6" t="s">
-        <v>1047</v>
+        <v>1031</v>
       </c>
       <c r="G185" s="8" t="s">
-        <v>1048</v>
+        <v>1032</v>
       </c>
     </row>
     <row r="186" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8908,10 +8908,10 @@
         <v>138</v>
       </c>
       <c r="F186" s="6" t="s">
-        <v>1049</v>
+        <v>1033</v>
       </c>
       <c r="G186" s="8" t="s">
-        <v>1050</v>
+        <v>1034</v>
       </c>
     </row>
     <row r="187" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8931,10 +8931,10 @@
         <v>138</v>
       </c>
       <c r="F187" s="6" t="s">
-        <v>1051</v>
+        <v>1035</v>
       </c>
       <c r="G187" s="8" t="s">
-        <v>1052</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="188" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8954,10 +8954,10 @@
         <v>138</v>
       </c>
       <c r="F188" s="6" t="s">
-        <v>1053</v>
+        <v>1037</v>
       </c>
       <c r="G188" s="8" t="s">
-        <v>1054</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="189" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8977,10 +8977,10 @@
         <v>138</v>
       </c>
       <c r="F189" s="6" t="s">
-        <v>1055</v>
+        <v>1039</v>
       </c>
       <c r="G189" s="8" t="s">
-        <v>1056</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="190" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9000,10 +9000,10 @@
         <v>138</v>
       </c>
       <c r="F190" s="6" t="s">
-        <v>1057</v>
+        <v>1041</v>
       </c>
       <c r="G190" s="8" t="s">
-        <v>1058</v>
+        <v>1042</v>
       </c>
     </row>
     <row r="191" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9023,10 +9023,10 @@
         <v>138</v>
       </c>
       <c r="F191" s="6" t="s">
-        <v>1059</v>
+        <v>1043</v>
       </c>
       <c r="G191" s="8" t="s">
-        <v>1060</v>
+        <v>1044</v>
       </c>
     </row>
     <row r="192" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9046,10 +9046,10 @@
         <v>138</v>
       </c>
       <c r="F192" s="6" t="s">
-        <v>1061</v>
+        <v>1045</v>
       </c>
       <c r="G192" s="8" t="s">
-        <v>1062</v>
+        <v>1046</v>
       </c>
     </row>
     <row r="193" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9069,10 +9069,10 @@
         <v>138</v>
       </c>
       <c r="F193" s="6" t="s">
-        <v>1063</v>
+        <v>1047</v>
       </c>
       <c r="G193" s="8" t="s">
-        <v>1064</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="194" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9092,10 +9092,10 @@
         <v>138</v>
       </c>
       <c r="F194" s="6" t="s">
-        <v>1065</v>
+        <v>1049</v>
       </c>
       <c r="G194" s="8" t="s">
-        <v>1066</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="195" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9115,10 +9115,10 @@
         <v>138</v>
       </c>
       <c r="F195" s="6" t="s">
-        <v>1067</v>
+        <v>1051</v>
       </c>
       <c r="G195" s="8" t="s">
-        <v>1068</v>
+        <v>1052</v>
       </c>
     </row>
     <row r="196" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9138,10 +9138,10 @@
         <v>138</v>
       </c>
       <c r="F196" s="6" t="s">
-        <v>1069</v>
+        <v>1053</v>
       </c>
       <c r="G196" s="8" t="s">
-        <v>1070</v>
+        <v>1054</v>
       </c>
     </row>
     <row r="197" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9161,10 +9161,10 @@
         <v>138</v>
       </c>
       <c r="F197" s="6" t="s">
-        <v>1071</v>
+        <v>1055</v>
       </c>
       <c r="G197" s="8" t="s">
-        <v>1072</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="198" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9184,10 +9184,10 @@
         <v>138</v>
       </c>
       <c r="F198" s="6" t="s">
-        <v>1073</v>
+        <v>1057</v>
       </c>
       <c r="G198" s="8" t="s">
-        <v>1074</v>
+        <v>1058</v>
       </c>
     </row>
     <row r="199" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9207,10 +9207,10 @@
         <v>138</v>
       </c>
       <c r="F199" s="6" t="s">
-        <v>1075</v>
+        <v>1059</v>
       </c>
       <c r="G199" s="8" t="s">
-        <v>1076</v>
+        <v>1060</v>
       </c>
     </row>
     <row r="200" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9230,10 +9230,10 @@
         <v>138</v>
       </c>
       <c r="F200" s="6" t="s">
-        <v>1077</v>
+        <v>1061</v>
       </c>
       <c r="G200" s="8" t="s">
-        <v>1078</v>
+        <v>1062</v>
       </c>
     </row>
     <row r="201" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9253,10 +9253,10 @@
         <v>138</v>
       </c>
       <c r="F201" s="6" t="s">
-        <v>1079</v>
+        <v>1063</v>
       </c>
       <c r="G201" s="8" t="s">
-        <v>1080</v>
+        <v>1064</v>
       </c>
     </row>
     <row r="202" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9276,10 +9276,10 @@
         <v>138</v>
       </c>
       <c r="F202" s="6" t="s">
-        <v>1081</v>
+        <v>1065</v>
       </c>
       <c r="G202" s="8" t="s">
-        <v>1082</v>
+        <v>1066</v>
       </c>
     </row>
     <row r="203" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9299,10 +9299,10 @@
         <v>138</v>
       </c>
       <c r="F203" s="6" t="s">
-        <v>1083</v>
+        <v>1067</v>
       </c>
       <c r="G203" s="8" t="s">
-        <v>1084</v>
+        <v>1068</v>
       </c>
     </row>
     <row r="204" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9322,10 +9322,10 @@
         <v>138</v>
       </c>
       <c r="F204" s="6" t="s">
-        <v>1085</v>
+        <v>1069</v>
       </c>
       <c r="G204" s="8" t="s">
-        <v>1086</v>
+        <v>1070</v>
       </c>
     </row>
     <row r="205" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9345,10 +9345,10 @@
         <v>138</v>
       </c>
       <c r="F205" s="6" t="s">
-        <v>1087</v>
+        <v>1071</v>
       </c>
       <c r="G205" s="8" t="s">
-        <v>1088</v>
+        <v>1072</v>
       </c>
     </row>
     <row r="206" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9368,10 +9368,10 @@
         <v>138</v>
       </c>
       <c r="F206" s="6" t="s">
-        <v>1089</v>
+        <v>1073</v>
       </c>
       <c r="G206" s="8" t="s">
-        <v>1090</v>
+        <v>1074</v>
       </c>
     </row>
     <row r="207" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9391,10 +9391,10 @@
         <v>138</v>
       </c>
       <c r="F207" s="6" t="s">
-        <v>1091</v>
+        <v>1075</v>
       </c>
       <c r="G207" s="8" t="s">
-        <v>1092</v>
+        <v>1076</v>
       </c>
     </row>
     <row r="208" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9414,10 +9414,10 @@
         <v>138</v>
       </c>
       <c r="F208" s="6" t="s">
-        <v>1093</v>
+        <v>1077</v>
       </c>
       <c r="G208" s="8" t="s">
-        <v>1094</v>
+        <v>1078</v>
       </c>
     </row>
     <row r="209" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9437,10 +9437,10 @@
         <v>138</v>
       </c>
       <c r="F209" s="6" t="s">
-        <v>1095</v>
+        <v>1079</v>
       </c>
       <c r="G209" s="8" t="s">
-        <v>1096</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="210" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9460,10 +9460,10 @@
         <v>138</v>
       </c>
       <c r="F210" s="6" t="s">
-        <v>1097</v>
+        <v>1081</v>
       </c>
       <c r="G210" s="8" t="s">
-        <v>1098</v>
+        <v>1082</v>
       </c>
     </row>
     <row r="211" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9483,10 +9483,10 @@
         <v>138</v>
       </c>
       <c r="F211" s="6" t="s">
-        <v>1099</v>
+        <v>1083</v>
       </c>
       <c r="G211" s="8" t="s">
-        <v>1100</v>
+        <v>1084</v>
       </c>
     </row>
     <row r="212" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9506,10 +9506,10 @@
         <v>138</v>
       </c>
       <c r="F212" s="6" t="s">
-        <v>1101</v>
+        <v>1085</v>
       </c>
       <c r="G212" s="8" t="s">
-        <v>1102</v>
+        <v>1086</v>
       </c>
     </row>
     <row r="213" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9529,10 +9529,10 @@
         <v>138</v>
       </c>
       <c r="F213" s="6" t="s">
-        <v>1103</v>
+        <v>1087</v>
       </c>
       <c r="G213" s="8" t="s">
-        <v>1104</v>
+        <v>1088</v>
       </c>
     </row>
     <row r="214" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9552,10 +9552,10 @@
         <v>138</v>
       </c>
       <c r="F214" s="6" t="s">
-        <v>1105</v>
+        <v>1089</v>
       </c>
       <c r="G214" s="8" t="s">
-        <v>1106</v>
+        <v>1090</v>
       </c>
     </row>
     <row r="215" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9575,10 +9575,10 @@
         <v>138</v>
       </c>
       <c r="F215" s="6" t="s">
-        <v>1107</v>
+        <v>1091</v>
       </c>
       <c r="G215" s="8" t="s">
-        <v>1108</v>
+        <v>1092</v>
       </c>
     </row>
     <row r="216" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9598,10 +9598,10 @@
         <v>138</v>
       </c>
       <c r="F216" s="6" t="s">
-        <v>1109</v>
+        <v>1093</v>
       </c>
       <c r="G216" s="8" t="s">
-        <v>1110</v>
+        <v>1094</v>
       </c>
     </row>
     <row r="217" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9621,10 +9621,10 @@
         <v>138</v>
       </c>
       <c r="F217" s="6" t="s">
-        <v>1111</v>
+        <v>1095</v>
       </c>
       <c r="G217" s="8" t="s">
-        <v>1112</v>
+        <v>1096</v>
       </c>
     </row>
     <row r="218" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9644,10 +9644,10 @@
         <v>138</v>
       </c>
       <c r="F218" s="6" t="s">
-        <v>1113</v>
+        <v>1097</v>
       </c>
       <c r="G218" s="8" t="s">
-        <v>1114</v>
+        <v>1098</v>
       </c>
     </row>
     <row r="219" spans="1:7" x14ac:dyDescent="0.3">
@@ -9667,10 +9667,10 @@
         <v>138</v>
       </c>
       <c r="F219" s="9" t="s">
-        <v>1115</v>
+        <v>1099</v>
       </c>
       <c r="G219" s="10" t="s">
-        <v>1116</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="220" spans="1:7" x14ac:dyDescent="0.3">
@@ -9690,10 +9690,10 @@
         <v>138</v>
       </c>
       <c r="F220" s="11" t="s">
-        <v>1117</v>
+        <v>1101</v>
       </c>
       <c r="G220" s="11" t="s">
-        <v>1118</v>
+        <v>1102</v>
       </c>
     </row>
     <row r="221" spans="1:7" x14ac:dyDescent="0.3">
@@ -9713,10 +9713,10 @@
         <v>138</v>
       </c>
       <c r="F221" s="11" t="s">
-        <v>1119</v>
+        <v>1103</v>
       </c>
       <c r="G221" s="11" t="s">
-        <v>1120</v>
+        <v>1104</v>
       </c>
     </row>
     <row r="222" spans="1:7" x14ac:dyDescent="0.3">
@@ -9736,10 +9736,10 @@
         <v>138</v>
       </c>
       <c r="F222" s="11" t="s">
-        <v>1121</v>
+        <v>1105</v>
       </c>
       <c r="G222" s="11" t="s">
-        <v>1122</v>
+        <v>1106</v>
       </c>
     </row>
     <row r="223" spans="1:7" x14ac:dyDescent="0.3">
@@ -9759,10 +9759,10 @@
         <v>138</v>
       </c>
       <c r="F223" s="11" t="s">
-        <v>1123</v>
+        <v>1107</v>
       </c>
       <c r="G223" s="11" t="s">
-        <v>1124</v>
+        <v>1108</v>
       </c>
     </row>
     <row r="224" spans="1:7" x14ac:dyDescent="0.3">
@@ -9782,10 +9782,10 @@
         <v>138</v>
       </c>
       <c r="F224" s="11" t="s">
-        <v>1125</v>
+        <v>1109</v>
       </c>
       <c r="G224" s="11" t="s">
-        <v>1126</v>
+        <v>1110</v>
       </c>
     </row>
     <row r="225" spans="1:7" x14ac:dyDescent="0.3">
@@ -9805,10 +9805,10 @@
         <v>138</v>
       </c>
       <c r="F225" s="11" t="s">
-        <v>1127</v>
+        <v>1111</v>
       </c>
       <c r="G225" s="11" t="s">
-        <v>1128</v>
+        <v>1112</v>
       </c>
     </row>
     <row r="226" spans="1:7" x14ac:dyDescent="0.3">
@@ -9828,10 +9828,10 @@
         <v>138</v>
       </c>
       <c r="F226" s="11" t="s">
-        <v>1129</v>
+        <v>1113</v>
       </c>
       <c r="G226" s="11" t="s">
-        <v>1130</v>
+        <v>1114</v>
       </c>
     </row>
     <row r="227" spans="1:7" x14ac:dyDescent="0.3">
@@ -9851,10 +9851,10 @@
         <v>138</v>
       </c>
       <c r="F227" s="11" t="s">
-        <v>1131</v>
+        <v>1115</v>
       </c>
       <c r="G227" s="11" t="s">
-        <v>1132</v>
+        <v>1116</v>
       </c>
     </row>
     <row r="228" spans="1:7" x14ac:dyDescent="0.3">
@@ -9874,10 +9874,10 @@
         <v>138</v>
       </c>
       <c r="F228" s="11" t="s">
-        <v>1133</v>
+        <v>1117</v>
       </c>
       <c r="G228" s="11" t="s">
-        <v>1134</v>
+        <v>1118</v>
       </c>
     </row>
     <row r="229" spans="1:7" x14ac:dyDescent="0.3">
@@ -9897,10 +9897,10 @@
         <v>138</v>
       </c>
       <c r="F229" s="11" t="s">
-        <v>1135</v>
+        <v>1119</v>
       </c>
       <c r="G229" s="11" t="s">
-        <v>1136</v>
+        <v>1120</v>
       </c>
     </row>
     <row r="230" spans="1:7" x14ac:dyDescent="0.3">
@@ -9920,10 +9920,10 @@
         <v>138</v>
       </c>
       <c r="F230" s="11" t="s">
-        <v>1137</v>
+        <v>1121</v>
       </c>
       <c r="G230" s="11" t="s">
-        <v>1138</v>
+        <v>1122</v>
       </c>
     </row>
     <row r="231" spans="1:7" x14ac:dyDescent="0.3">
@@ -9943,10 +9943,10 @@
         <v>138</v>
       </c>
       <c r="F231" s="11" t="s">
-        <v>1139</v>
+        <v>1123</v>
       </c>
       <c r="G231" s="11" t="s">
-        <v>1140</v>
+        <v>1124</v>
       </c>
     </row>
     <row r="232" spans="1:7" x14ac:dyDescent="0.3">
@@ -9966,10 +9966,10 @@
         <v>138</v>
       </c>
       <c r="F232" s="11" t="s">
-        <v>1141</v>
+        <v>1125</v>
       </c>
       <c r="G232" s="11" t="s">
-        <v>1142</v>
+        <v>1126</v>
       </c>
     </row>
     <row r="233" spans="1:7" x14ac:dyDescent="0.3">
@@ -9989,10 +9989,10 @@
         <v>138</v>
       </c>
       <c r="F233" s="11" t="s">
-        <v>1143</v>
+        <v>1127</v>
       </c>
       <c r="G233" s="11" t="s">
-        <v>1144</v>
+        <v>1128</v>
       </c>
     </row>
     <row r="234" spans="1:7" x14ac:dyDescent="0.3">
@@ -10012,10 +10012,10 @@
         <v>138</v>
       </c>
       <c r="F234" s="11" t="s">
-        <v>1145</v>
+        <v>1129</v>
       </c>
       <c r="G234" s="11" t="s">
-        <v>1146</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="235" spans="1:7" x14ac:dyDescent="0.3">
@@ -10035,10 +10035,10 @@
         <v>138</v>
       </c>
       <c r="F235" s="11" t="s">
-        <v>1147</v>
+        <v>1131</v>
       </c>
       <c r="G235" s="11" t="s">
-        <v>1148</v>
+        <v>1132</v>
       </c>
     </row>
     <row r="236" spans="1:7" x14ac:dyDescent="0.3">
@@ -10058,10 +10058,10 @@
         <v>138</v>
       </c>
       <c r="F236" s="11" t="s">
-        <v>1149</v>
+        <v>1133</v>
       </c>
       <c r="G236" s="11" t="s">
-        <v>1150</v>
+        <v>1134</v>
       </c>
     </row>
     <row r="237" spans="1:7" x14ac:dyDescent="0.3">
@@ -10081,10 +10081,10 @@
         <v>138</v>
       </c>
       <c r="F237" s="11" t="s">
-        <v>1151</v>
+        <v>1135</v>
       </c>
       <c r="G237" s="11" t="s">
-        <v>1152</v>
+        <v>1136</v>
       </c>
     </row>
     <row r="238" spans="1:7" x14ac:dyDescent="0.3">
@@ -10104,10 +10104,10 @@
         <v>138</v>
       </c>
       <c r="F238" s="11" t="s">
-        <v>1153</v>
+        <v>1137</v>
       </c>
       <c r="G238" s="11" t="s">
-        <v>1154</v>
+        <v>1138</v>
       </c>
     </row>
     <row r="239" spans="1:7" x14ac:dyDescent="0.3">
@@ -10127,10 +10127,10 @@
         <v>138</v>
       </c>
       <c r="F239" s="11" t="s">
-        <v>1155</v>
+        <v>1139</v>
       </c>
       <c r="G239" s="11" t="s">
-        <v>1156</v>
+        <v>1140</v>
       </c>
     </row>
     <row r="240" spans="1:7" x14ac:dyDescent="0.3">
@@ -10150,10 +10150,10 @@
         <v>138</v>
       </c>
       <c r="F240" s="11" t="s">
-        <v>1157</v>
+        <v>1141</v>
       </c>
       <c r="G240" s="11" t="s">
-        <v>1158</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="241" spans="1:7" x14ac:dyDescent="0.3">
@@ -10173,10 +10173,10 @@
         <v>138</v>
       </c>
       <c r="F241" s="11" t="s">
-        <v>1159</v>
+        <v>1143</v>
       </c>
       <c r="G241" s="11" t="s">
-        <v>1160</v>
+        <v>1144</v>
       </c>
     </row>
     <row r="242" spans="1:7" x14ac:dyDescent="0.3">
@@ -10196,10 +10196,10 @@
         <v>138</v>
       </c>
       <c r="F242" s="11" t="s">
-        <v>1161</v>
+        <v>1145</v>
       </c>
       <c r="G242" s="11" t="s">
-        <v>1162</v>
+        <v>1146</v>
       </c>
     </row>
     <row r="243" spans="1:7" x14ac:dyDescent="0.3">
@@ -10219,10 +10219,10 @@
         <v>138</v>
       </c>
       <c r="F243" s="11" t="s">
-        <v>1163</v>
+        <v>1147</v>
       </c>
       <c r="G243" s="11" t="s">
-        <v>1164</v>
+        <v>1148</v>
       </c>
     </row>
     <row r="244" spans="1:7" x14ac:dyDescent="0.3">
@@ -10242,10 +10242,10 @@
         <v>138</v>
       </c>
       <c r="F244" s="11" t="s">
-        <v>1165</v>
+        <v>1149</v>
       </c>
       <c r="G244" s="11" t="s">
-        <v>1166</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="245" spans="1:7" x14ac:dyDescent="0.3">
@@ -10265,10 +10265,10 @@
         <v>138</v>
       </c>
       <c r="F245" s="11" t="s">
-        <v>1167</v>
+        <v>1151</v>
       </c>
       <c r="G245" s="11" t="s">
-        <v>1168</v>
+        <v>1152</v>
       </c>
     </row>
     <row r="246" spans="1:7" x14ac:dyDescent="0.3">
@@ -10288,10 +10288,10 @@
         <v>138</v>
       </c>
       <c r="F246" s="11" t="s">
-        <v>1169</v>
+        <v>1153</v>
       </c>
       <c r="G246" s="11" t="s">
-        <v>1170</v>
+        <v>1154</v>
       </c>
     </row>
     <row r="247" spans="1:7" x14ac:dyDescent="0.3">
@@ -10311,10 +10311,10 @@
         <v>138</v>
       </c>
       <c r="F247" s="11" t="s">
-        <v>1171</v>
+        <v>1155</v>
       </c>
       <c r="G247" s="11" t="s">
-        <v>1172</v>
+        <v>1156</v>
       </c>
     </row>
     <row r="248" spans="1:7" x14ac:dyDescent="0.3">
@@ -10334,10 +10334,10 @@
         <v>138</v>
       </c>
       <c r="F248" s="11" t="s">
-        <v>1173</v>
+        <v>1157</v>
       </c>
       <c r="G248" s="11" t="s">
-        <v>1174</v>
+        <v>1158</v>
       </c>
     </row>
     <row r="249" spans="1:7" x14ac:dyDescent="0.3">
@@ -10357,10 +10357,10 @@
         <v>138</v>
       </c>
       <c r="F249" s="11" t="s">
-        <v>1175</v>
+        <v>1159</v>
       </c>
       <c r="G249" s="11" t="s">
-        <v>1176</v>
+        <v>1160</v>
       </c>
     </row>
     <row r="250" spans="1:7" x14ac:dyDescent="0.3">
@@ -10380,10 +10380,10 @@
         <v>138</v>
       </c>
       <c r="F250" s="11" t="s">
-        <v>1177</v>
+        <v>1161</v>
       </c>
       <c r="G250" s="11" t="s">
-        <v>1178</v>
+        <v>1162</v>
       </c>
     </row>
     <row r="251" spans="1:7" x14ac:dyDescent="0.3">
@@ -10403,10 +10403,10 @@
         <v>138</v>
       </c>
       <c r="F251" s="11" t="s">
-        <v>1179</v>
+        <v>1163</v>
       </c>
       <c r="G251" s="11" t="s">
-        <v>1180</v>
+        <v>1164</v>
       </c>
     </row>
     <row r="252" spans="1:7" x14ac:dyDescent="0.3">
@@ -10426,10 +10426,10 @@
         <v>138</v>
       </c>
       <c r="F252" s="11" t="s">
-        <v>1181</v>
+        <v>1165</v>
       </c>
       <c r="G252" s="11" t="s">
-        <v>1182</v>
+        <v>1166</v>
       </c>
     </row>
     <row r="253" spans="1:7" x14ac:dyDescent="0.3">
@@ -10449,10 +10449,10 @@
         <v>138</v>
       </c>
       <c r="F253" s="11" t="s">
-        <v>1183</v>
+        <v>1167</v>
       </c>
       <c r="G253" s="11" t="s">
-        <v>1184</v>
+        <v>1168</v>
       </c>
     </row>
     <row r="254" spans="1:7" x14ac:dyDescent="0.3">
@@ -10472,10 +10472,10 @@
         <v>138</v>
       </c>
       <c r="F254" s="11" t="s">
-        <v>1185</v>
+        <v>1169</v>
       </c>
       <c r="G254" s="11" t="s">
-        <v>1186</v>
+        <v>1170</v>
       </c>
     </row>
     <row r="255" spans="1:7" x14ac:dyDescent="0.3">
@@ -10495,10 +10495,10 @@
         <v>138</v>
       </c>
       <c r="F255" s="11" t="s">
-        <v>1187</v>
+        <v>1171</v>
       </c>
       <c r="G255" s="11" t="s">
-        <v>1188</v>
+        <v>1172</v>
       </c>
     </row>
     <row r="256" spans="1:7" x14ac:dyDescent="0.3">
@@ -10518,10 +10518,10 @@
         <v>138</v>
       </c>
       <c r="F256" s="11" t="s">
-        <v>1189</v>
+        <v>1173</v>
       </c>
       <c r="G256" s="11" t="s">
-        <v>1190</v>
+        <v>1174</v>
       </c>
     </row>
     <row r="257" spans="1:7" x14ac:dyDescent="0.3">
@@ -10541,10 +10541,10 @@
         <v>138</v>
       </c>
       <c r="F257" s="11" t="s">
-        <v>1191</v>
+        <v>1175</v>
       </c>
       <c r="G257" s="11" t="s">
-        <v>1192</v>
+        <v>1176</v>
       </c>
     </row>
     <row r="258" spans="1:7" x14ac:dyDescent="0.3">
@@ -10564,10 +10564,10 @@
         <v>138</v>
       </c>
       <c r="F258" s="11" t="s">
-        <v>1193</v>
+        <v>1177</v>
       </c>
       <c r="G258" s="11" t="s">
-        <v>1194</v>
+        <v>1178</v>
       </c>
     </row>
     <row r="259" spans="1:7" x14ac:dyDescent="0.3">
@@ -10587,10 +10587,10 @@
         <v>138</v>
       </c>
       <c r="F259" s="11" t="s">
-        <v>1195</v>
+        <v>1179</v>
       </c>
       <c r="G259" s="11" t="s">
-        <v>1196</v>
+        <v>1180</v>
       </c>
     </row>
     <row r="260" spans="1:7" x14ac:dyDescent="0.3">
@@ -10610,10 +10610,10 @@
         <v>138</v>
       </c>
       <c r="F260" s="11" t="s">
-        <v>1197</v>
+        <v>1181</v>
       </c>
       <c r="G260" s="11" t="s">
-        <v>1198</v>
+        <v>1182</v>
       </c>
     </row>
     <row r="261" spans="1:7" x14ac:dyDescent="0.3">
@@ -10633,10 +10633,10 @@
         <v>138</v>
       </c>
       <c r="F261" s="11" t="s">
-        <v>1199</v>
+        <v>1183</v>
       </c>
       <c r="G261" s="11" t="s">
-        <v>1200</v>
+        <v>1184</v>
       </c>
     </row>
     <row r="262" spans="1:7" x14ac:dyDescent="0.3">
@@ -10656,10 +10656,10 @@
         <v>138</v>
       </c>
       <c r="F262" s="11" t="s">
-        <v>1201</v>
+        <v>1185</v>
       </c>
       <c r="G262" s="11" t="s">
-        <v>1202</v>
+        <v>1186</v>
       </c>
     </row>
     <row r="263" spans="1:7" x14ac:dyDescent="0.3">
@@ -10679,10 +10679,10 @@
         <v>138</v>
       </c>
       <c r="F263" s="11" t="s">
-        <v>1203</v>
+        <v>1187</v>
       </c>
       <c r="G263" s="11" t="s">
-        <v>1204</v>
+        <v>1188</v>
       </c>
     </row>
     <row r="264" spans="1:7" x14ac:dyDescent="0.3">
@@ -10702,10 +10702,10 @@
         <v>138</v>
       </c>
       <c r="F264" s="11" t="s">
-        <v>1205</v>
+        <v>1189</v>
       </c>
       <c r="G264" s="11" t="s">
-        <v>1206</v>
+        <v>1190</v>
       </c>
     </row>
     <row r="265" spans="1:7" x14ac:dyDescent="0.3">
@@ -10725,10 +10725,10 @@
         <v>138</v>
       </c>
       <c r="F265" s="11" t="s">
-        <v>1207</v>
+        <v>1191</v>
       </c>
       <c r="G265" s="11" t="s">
-        <v>1208</v>
+        <v>1192</v>
       </c>
     </row>
     <row r="266" spans="1:7" x14ac:dyDescent="0.3">
@@ -10748,10 +10748,10 @@
         <v>138</v>
       </c>
       <c r="F266" s="11" t="s">
-        <v>1209</v>
+        <v>1193</v>
       </c>
       <c r="G266" s="11" t="s">
-        <v>1210</v>
+        <v>1194</v>
       </c>
     </row>
     <row r="267" spans="1:7" x14ac:dyDescent="0.3">
@@ -10771,10 +10771,10 @@
         <v>138</v>
       </c>
       <c r="F267" s="11" t="s">
-        <v>1211</v>
+        <v>1195</v>
       </c>
       <c r="G267" s="11" t="s">
-        <v>1212</v>
+        <v>1196</v>
       </c>
     </row>
     <row r="268" spans="1:7" x14ac:dyDescent="0.3">
@@ -10794,10 +10794,10 @@
         <v>138</v>
       </c>
       <c r="F268" s="11" t="s">
-        <v>1213</v>
+        <v>1197</v>
       </c>
       <c r="G268" s="11" t="s">
-        <v>1214</v>
+        <v>1198</v>
       </c>
     </row>
     <row r="269" spans="1:7" x14ac:dyDescent="0.3">
@@ -10817,10 +10817,10 @@
         <v>138</v>
       </c>
       <c r="F269" s="11" t="s">
-        <v>1215</v>
+        <v>1199</v>
       </c>
       <c r="G269" s="11" t="s">
-        <v>1216</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="270" spans="1:7" x14ac:dyDescent="0.3">
@@ -10840,10 +10840,10 @@
         <v>138</v>
       </c>
       <c r="F270" s="11" t="s">
-        <v>1217</v>
+        <v>1201</v>
       </c>
       <c r="G270" s="11" t="s">
-        <v>1218</v>
+        <v>1202</v>
       </c>
     </row>
     <row r="271" spans="1:7" x14ac:dyDescent="0.3">
@@ -10863,10 +10863,10 @@
         <v>138</v>
       </c>
       <c r="F271" s="11" t="s">
-        <v>1219</v>
+        <v>1203</v>
       </c>
       <c r="G271" s="11" t="s">
-        <v>1220</v>
+        <v>1204</v>
       </c>
     </row>
     <row r="272" spans="1:7" x14ac:dyDescent="0.3">
@@ -10886,10 +10886,10 @@
         <v>138</v>
       </c>
       <c r="F272" s="11" t="s">
-        <v>1221</v>
+        <v>1205</v>
       </c>
       <c r="G272" s="11" t="s">
-        <v>1222</v>
+        <v>1206</v>
       </c>
     </row>
     <row r="273" spans="1:7" x14ac:dyDescent="0.3">
@@ -10909,10 +10909,10 @@
         <v>138</v>
       </c>
       <c r="F273" s="11" t="s">
-        <v>1223</v>
+        <v>1207</v>
       </c>
       <c r="G273" s="11" t="s">
-        <v>1224</v>
+        <v>1208</v>
       </c>
     </row>
     <row r="274" spans="1:7" x14ac:dyDescent="0.3">
@@ -10932,10 +10932,10 @@
         <v>138</v>
       </c>
       <c r="F274" s="11" t="s">
-        <v>1225</v>
+        <v>1209</v>
       </c>
       <c r="G274" s="11" t="s">
-        <v>1226</v>
+        <v>1210</v>
       </c>
     </row>
     <row r="275" spans="1:7" x14ac:dyDescent="0.3">
@@ -10955,10 +10955,10 @@
         <v>138</v>
       </c>
       <c r="F275" s="11" t="s">
-        <v>1227</v>
+        <v>1211</v>
       </c>
       <c r="G275" s="11" t="s">
-        <v>1228</v>
+        <v>1212</v>
       </c>
     </row>
     <row r="276" spans="1:7" x14ac:dyDescent="0.3">
@@ -10978,10 +10978,10 @@
         <v>138</v>
       </c>
       <c r="F276" s="11" t="s">
-        <v>1229</v>
+        <v>1213</v>
       </c>
       <c r="G276" s="11" t="s">
-        <v>1230</v>
+        <v>1214</v>
       </c>
     </row>
     <row r="277" spans="1:7" x14ac:dyDescent="0.3">
@@ -11001,10 +11001,10 @@
         <v>138</v>
       </c>
       <c r="F277" s="11" t="s">
-        <v>1231</v>
+        <v>1215</v>
       </c>
       <c r="G277" s="11" t="s">
-        <v>1232</v>
+        <v>1216</v>
       </c>
     </row>
     <row r="278" spans="1:7" x14ac:dyDescent="0.3">
@@ -11024,10 +11024,10 @@
         <v>138</v>
       </c>
       <c r="F278" s="11" t="s">
-        <v>1233</v>
+        <v>1217</v>
       </c>
       <c r="G278" s="11" t="s">
-        <v>1234</v>
+        <v>1218</v>
       </c>
     </row>
     <row r="279" spans="1:7" x14ac:dyDescent="0.3">
@@ -11047,10 +11047,10 @@
         <v>138</v>
       </c>
       <c r="F279" s="11" t="s">
-        <v>1235</v>
+        <v>1219</v>
       </c>
       <c r="G279" s="11" t="s">
-        <v>1236</v>
+        <v>1220</v>
       </c>
     </row>
     <row r="280" spans="1:7" x14ac:dyDescent="0.3">
@@ -11070,10 +11070,10 @@
         <v>138</v>
       </c>
       <c r="F280" s="11" t="s">
-        <v>1237</v>
+        <v>1221</v>
       </c>
       <c r="G280" s="11" t="s">
-        <v>1238</v>
+        <v>1222</v>
       </c>
     </row>
     <row r="281" spans="1:7" x14ac:dyDescent="0.3">
@@ -11093,10 +11093,10 @@
         <v>138</v>
       </c>
       <c r="F281" s="11" t="s">
-        <v>1239</v>
+        <v>1223</v>
       </c>
       <c r="G281" s="11" t="s">
-        <v>1240</v>
+        <v>1224</v>
       </c>
     </row>
     <row r="282" spans="1:7" x14ac:dyDescent="0.3">
@@ -11116,10 +11116,10 @@
         <v>603</v>
       </c>
       <c r="F282" s="11" t="s">
-        <v>1241</v>
+        <v>1225</v>
       </c>
       <c r="G282" s="11" t="s">
-        <v>1242</v>
+        <v>1226</v>
       </c>
     </row>
     <row r="283" spans="1:7" x14ac:dyDescent="0.3">
@@ -11139,10 +11139,10 @@
         <v>603</v>
       </c>
       <c r="F283" s="11" t="s">
-        <v>1243</v>
+        <v>1227</v>
       </c>
       <c r="G283" s="11" t="s">
-        <v>1244</v>
+        <v>1228</v>
       </c>
     </row>
     <row r="284" spans="1:7" x14ac:dyDescent="0.3">
@@ -11162,10 +11162,10 @@
         <v>603</v>
       </c>
       <c r="F284" s="11" t="s">
-        <v>1245</v>
+        <v>1229</v>
       </c>
       <c r="G284" s="11" t="s">
-        <v>1246</v>
+        <v>1230</v>
       </c>
     </row>
     <row r="285" spans="1:7" x14ac:dyDescent="0.3">
@@ -11185,10 +11185,10 @@
         <v>603</v>
       </c>
       <c r="F285" s="11" t="s">
-        <v>1247</v>
+        <v>1231</v>
       </c>
       <c r="G285" s="11" t="s">
-        <v>1248</v>
+        <v>1232</v>
       </c>
     </row>
     <row r="286" spans="1:7" x14ac:dyDescent="0.3">
@@ -11208,10 +11208,10 @@
         <v>603</v>
       </c>
       <c r="F286" s="11" t="s">
-        <v>1249</v>
+        <v>1233</v>
       </c>
       <c r="G286" s="11" t="s">
-        <v>1250</v>
+        <v>1234</v>
       </c>
     </row>
     <row r="287" spans="1:7" x14ac:dyDescent="0.3">
@@ -11231,10 +11231,10 @@
         <v>603</v>
       </c>
       <c r="F287" s="11" t="s">
-        <v>1251</v>
+        <v>1235</v>
       </c>
       <c r="G287" s="11" t="s">
-        <v>1252</v>
+        <v>1236</v>
       </c>
     </row>
     <row r="288" spans="1:7" x14ac:dyDescent="0.3">
@@ -11254,10 +11254,10 @@
         <v>603</v>
       </c>
       <c r="F288" s="11" t="s">
-        <v>1253</v>
+        <v>1237</v>
       </c>
       <c r="G288" s="11" t="s">
-        <v>1254</v>
+        <v>1238</v>
       </c>
     </row>
     <row r="289" spans="1:7" x14ac:dyDescent="0.3">
@@ -11277,10 +11277,10 @@
         <v>603</v>
       </c>
       <c r="F289" s="11" t="s">
-        <v>1255</v>
+        <v>1239</v>
       </c>
       <c r="G289" s="11" t="s">
-        <v>1256</v>
+        <v>1240</v>
       </c>
     </row>
     <row r="290" spans="1:7" x14ac:dyDescent="0.3">
@@ -11300,10 +11300,10 @@
         <v>603</v>
       </c>
       <c r="F290" s="11" t="s">
-        <v>1257</v>
+        <v>1241</v>
       </c>
       <c r="G290" s="11" t="s">
-        <v>1258</v>
+        <v>1242</v>
       </c>
     </row>
     <row r="291" spans="1:7" x14ac:dyDescent="0.3">
@@ -11323,10 +11323,10 @@
         <v>603</v>
       </c>
       <c r="F291" s="11" t="s">
-        <v>1259</v>
+        <v>1243</v>
       </c>
       <c r="G291" s="11" t="s">
-        <v>1260</v>
+        <v>1244</v>
       </c>
     </row>
     <row r="292" spans="1:7" x14ac:dyDescent="0.3">
@@ -11346,10 +11346,10 @@
         <v>603</v>
       </c>
       <c r="F292" s="11" t="s">
-        <v>1261</v>
+        <v>1245</v>
       </c>
       <c r="G292" s="11" t="s">
-        <v>1262</v>
+        <v>1246</v>
       </c>
     </row>
     <row r="293" spans="1:7" x14ac:dyDescent="0.3">
@@ -11369,10 +11369,10 @@
         <v>603</v>
       </c>
       <c r="F293" s="11" t="s">
-        <v>1263</v>
+        <v>1247</v>
       </c>
       <c r="G293" s="11" t="s">
-        <v>1264</v>
+        <v>1248</v>
       </c>
     </row>
     <row r="294" spans="1:7" x14ac:dyDescent="0.3">
@@ -11392,10 +11392,10 @@
         <v>603</v>
       </c>
       <c r="F294" s="11" t="s">
-        <v>1265</v>
+        <v>1249</v>
       </c>
       <c r="G294" s="11" t="s">
-        <v>1266</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="295" spans="1:7" x14ac:dyDescent="0.3">
@@ -11415,10 +11415,10 @@
         <v>603</v>
       </c>
       <c r="F295" s="11" t="s">
-        <v>1267</v>
+        <v>1251</v>
       </c>
       <c r="G295" s="11" t="s">
-        <v>1268</v>
+        <v>1252</v>
       </c>
     </row>
     <row r="296" spans="1:7" x14ac:dyDescent="0.3">
@@ -11438,10 +11438,10 @@
         <v>603</v>
       </c>
       <c r="F296" s="11" t="s">
-        <v>1269</v>
+        <v>1253</v>
       </c>
       <c r="G296" s="11" t="s">
-        <v>1270</v>
+        <v>1254</v>
       </c>
     </row>
     <row r="297" spans="1:7" x14ac:dyDescent="0.3">
@@ -11461,10 +11461,10 @@
         <v>603</v>
       </c>
       <c r="F297" s="11" t="s">
-        <v>1271</v>
+        <v>1255</v>
       </c>
       <c r="G297" s="11" t="s">
-        <v>1272</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="298" spans="1:7" x14ac:dyDescent="0.3">
@@ -11484,10 +11484,10 @@
         <v>138</v>
       </c>
       <c r="F298" s="11" t="s">
-        <v>1273</v>
+        <v>1257</v>
       </c>
       <c r="G298" s="11" t="s">
-        <v>1274</v>
+        <v>1258</v>
       </c>
     </row>
     <row r="299" spans="1:7" x14ac:dyDescent="0.3">
@@ -11507,10 +11507,10 @@
         <v>138</v>
       </c>
       <c r="F299" s="11" t="s">
-        <v>1275</v>
+        <v>1259</v>
       </c>
       <c r="G299" s="11" t="s">
-        <v>1276</v>
+        <v>1260</v>
       </c>
     </row>
     <row r="300" spans="1:7" x14ac:dyDescent="0.3">
@@ -11530,10 +11530,10 @@
         <v>138</v>
       </c>
       <c r="F300" s="11" t="s">
-        <v>1277</v>
+        <v>1261</v>
       </c>
       <c r="G300" s="11" t="s">
-        <v>1278</v>
+        <v>1262</v>
       </c>
     </row>
     <row r="301" spans="1:7" x14ac:dyDescent="0.3">
@@ -11553,10 +11553,10 @@
         <v>138</v>
       </c>
       <c r="F301" s="11" t="s">
-        <v>1279</v>
+        <v>1263</v>
       </c>
       <c r="G301" s="11" t="s">
-        <v>1280</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="302" spans="1:7" x14ac:dyDescent="0.3">
@@ -11576,10 +11576,10 @@
         <v>138</v>
       </c>
       <c r="F302" s="11" t="s">
-        <v>1281</v>
+        <v>1265</v>
       </c>
       <c r="G302" s="11" t="s">
-        <v>1282</v>
+        <v>1266</v>
       </c>
     </row>
     <row r="303" spans="1:7" x14ac:dyDescent="0.3">
@@ -11599,10 +11599,10 @@
         <v>138</v>
       </c>
       <c r="F303" s="11" t="s">
-        <v>1283</v>
+        <v>1267</v>
       </c>
       <c r="G303" s="11" t="s">
-        <v>1284</v>
+        <v>1268</v>
       </c>
     </row>
     <row r="304" spans="1:7" x14ac:dyDescent="0.3">
@@ -11622,10 +11622,10 @@
         <v>138</v>
       </c>
       <c r="F304" s="11" t="s">
-        <v>1285</v>
+        <v>1269</v>
       </c>
       <c r="G304" s="11" t="s">
-        <v>1286</v>
+        <v>1270</v>
       </c>
     </row>
     <row r="305" spans="1:7" x14ac:dyDescent="0.3">
@@ -11645,10 +11645,10 @@
         <v>138</v>
       </c>
       <c r="F305" s="11" t="s">
-        <v>1287</v>
+        <v>1271</v>
       </c>
       <c r="G305" s="11" t="s">
-        <v>1288</v>
+        <v>1272</v>
       </c>
     </row>
     <row r="306" spans="1:7" x14ac:dyDescent="0.3">
@@ -11668,10 +11668,10 @@
         <v>138</v>
       </c>
       <c r="F306" s="11" t="s">
-        <v>1289</v>
+        <v>1273</v>
       </c>
       <c r="G306" s="11" t="s">
-        <v>1290</v>
+        <v>1274</v>
       </c>
     </row>
     <row r="307" spans="1:7" x14ac:dyDescent="0.3">
@@ -11691,10 +11691,10 @@
         <v>138</v>
       </c>
       <c r="F307" s="11" t="s">
-        <v>1291</v>
+        <v>1275</v>
       </c>
       <c r="G307" s="11" t="s">
-        <v>1292</v>
+        <v>1276</v>
       </c>
     </row>
     <row r="308" spans="1:7" x14ac:dyDescent="0.3">
@@ -11714,10 +11714,10 @@
         <v>603</v>
       </c>
       <c r="F308" s="11" t="s">
-        <v>1293</v>
+        <v>1277</v>
       </c>
       <c r="G308" s="11" t="s">
-        <v>1294</v>
+        <v>1278</v>
       </c>
     </row>
     <row r="309" spans="1:7" x14ac:dyDescent="0.3">
@@ -11737,10 +11737,10 @@
         <v>603</v>
       </c>
       <c r="F309" s="11" t="s">
-        <v>1295</v>
+        <v>1279</v>
       </c>
       <c r="G309" s="11" t="s">
-        <v>1296</v>
+        <v>1280</v>
       </c>
     </row>
     <row r="310" spans="1:7" x14ac:dyDescent="0.3">
@@ -11760,10 +11760,10 @@
         <v>603</v>
       </c>
       <c r="F310" s="11" t="s">
-        <v>1297</v>
+        <v>1281</v>
       </c>
       <c r="G310" s="11" t="s">
-        <v>1298</v>
+        <v>1282</v>
       </c>
     </row>
     <row r="311" spans="1:7" x14ac:dyDescent="0.3">
@@ -11783,10 +11783,10 @@
         <v>603</v>
       </c>
       <c r="F311" s="11" t="s">
-        <v>1299</v>
+        <v>1283</v>
       </c>
       <c r="G311" s="11" t="s">
-        <v>1300</v>
+        <v>1284</v>
       </c>
     </row>
     <row r="312" spans="1:7" x14ac:dyDescent="0.3">
@@ -11806,10 +11806,10 @@
         <v>603</v>
       </c>
       <c r="F312" s="11" t="s">
-        <v>1301</v>
+        <v>1285</v>
       </c>
       <c r="G312" s="11" t="s">
-        <v>1302</v>
+        <v>1286</v>
       </c>
     </row>
     <row r="313" spans="1:7" x14ac:dyDescent="0.3">
@@ -11829,10 +11829,10 @@
         <v>603</v>
       </c>
       <c r="F313" s="11" t="s">
-        <v>1303</v>
+        <v>1287</v>
       </c>
       <c r="G313" s="11" t="s">
-        <v>1304</v>
+        <v>1288</v>
       </c>
     </row>
     <row r="314" spans="1:7" x14ac:dyDescent="0.3">
@@ -11852,10 +11852,10 @@
         <v>603</v>
       </c>
       <c r="F314" s="11" t="s">
-        <v>1305</v>
+        <v>1289</v>
       </c>
       <c r="G314" s="11" t="s">
-        <v>1306</v>
+        <v>1290</v>
       </c>
     </row>
     <row r="315" spans="1:7" x14ac:dyDescent="0.3">
@@ -11875,10 +11875,10 @@
         <v>603</v>
       </c>
       <c r="F315" s="11" t="s">
-        <v>1307</v>
+        <v>1291</v>
       </c>
       <c r="G315" s="11" t="s">
-        <v>1308</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="316" spans="1:7" x14ac:dyDescent="0.3">
@@ -11898,10 +11898,10 @@
         <v>603</v>
       </c>
       <c r="F316" s="11" t="s">
-        <v>1309</v>
+        <v>1293</v>
       </c>
       <c r="G316" s="11" t="s">
-        <v>1310</v>
+        <v>1294</v>
       </c>
     </row>
     <row r="317" spans="1:7" x14ac:dyDescent="0.3">
@@ -11921,10 +11921,10 @@
         <v>603</v>
       </c>
       <c r="F317" s="11" t="s">
-        <v>1311</v>
+        <v>1295</v>
       </c>
       <c r="G317" s="11" t="s">
-        <v>1312</v>
+        <v>1296</v>
       </c>
     </row>
     <row r="318" spans="1:7" x14ac:dyDescent="0.3">
@@ -11944,10 +11944,10 @@
         <v>603</v>
       </c>
       <c r="F318" s="11" t="s">
-        <v>1313</v>
+        <v>1297</v>
       </c>
       <c r="G318" s="11" t="s">
-        <v>1314</v>
+        <v>1298</v>
       </c>
     </row>
     <row r="319" spans="1:7" x14ac:dyDescent="0.3">
@@ -11967,10 +11967,10 @@
         <v>603</v>
       </c>
       <c r="F319" s="11" t="s">
-        <v>1315</v>
+        <v>1299</v>
       </c>
       <c r="G319" s="11" t="s">
-        <v>1316</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="320" spans="1:7" x14ac:dyDescent="0.3">
@@ -11990,10 +11990,10 @@
         <v>603</v>
       </c>
       <c r="F320" s="11" t="s">
-        <v>1317</v>
+        <v>1301</v>
       </c>
       <c r="G320" s="11" t="s">
-        <v>1318</v>
+        <v>1302</v>
       </c>
     </row>
     <row r="321" spans="1:7" x14ac:dyDescent="0.3">
@@ -12013,10 +12013,10 @@
         <v>603</v>
       </c>
       <c r="F321" s="11" t="s">
-        <v>1319</v>
+        <v>1303</v>
       </c>
       <c r="G321" s="11" t="s">
-        <v>1320</v>
+        <v>1304</v>
       </c>
     </row>
     <row r="322" spans="1:7" x14ac:dyDescent="0.3">
@@ -12036,10 +12036,10 @@
         <v>603</v>
       </c>
       <c r="F322" s="11" t="s">
-        <v>1321</v>
+        <v>1305</v>
       </c>
       <c r="G322" s="11" t="s">
-        <v>1322</v>
+        <v>1306</v>
       </c>
     </row>
     <row r="323" spans="1:7" x14ac:dyDescent="0.3">
@@ -12059,10 +12059,10 @@
         <v>603</v>
       </c>
       <c r="F323" s="11" t="s">
-        <v>1323</v>
+        <v>1307</v>
       </c>
       <c r="G323" s="11" t="s">
-        <v>1324</v>
+        <v>1308</v>
       </c>
     </row>
     <row r="324" spans="1:7" x14ac:dyDescent="0.3">
@@ -12082,10 +12082,10 @@
         <v>603</v>
       </c>
       <c r="F324" s="11" t="s">
-        <v>1325</v>
+        <v>1309</v>
       </c>
       <c r="G324" s="11" t="s">
-        <v>1326</v>
+        <v>1310</v>
       </c>
     </row>
     <row r="325" spans="1:7" x14ac:dyDescent="0.3">
@@ -12105,10 +12105,10 @@
         <v>603</v>
       </c>
       <c r="F325" s="11" t="s">
-        <v>1327</v>
+        <v>1311</v>
       </c>
       <c r="G325" s="11" t="s">
-        <v>1328</v>
+        <v>1312</v>
       </c>
     </row>
     <row r="326" spans="1:7" x14ac:dyDescent="0.3">
@@ -12128,10 +12128,10 @@
         <v>603</v>
       </c>
       <c r="F326" s="11" t="s">
-        <v>1329</v>
+        <v>1313</v>
       </c>
       <c r="G326" s="11" t="s">
-        <v>1330</v>
+        <v>1314</v>
       </c>
     </row>
     <row r="327" spans="1:7" x14ac:dyDescent="0.3">
@@ -12151,10 +12151,10 @@
         <v>603</v>
       </c>
       <c r="F327" s="11" t="s">
-        <v>1331</v>
+        <v>1315</v>
       </c>
       <c r="G327" s="11" t="s">
-        <v>1332</v>
+        <v>1316</v>
       </c>
     </row>
     <row r="328" spans="1:7" x14ac:dyDescent="0.3">
@@ -12174,10 +12174,10 @@
         <v>603</v>
       </c>
       <c r="F328" s="11" t="s">
-        <v>1333</v>
+        <v>1317</v>
       </c>
       <c r="G328" s="11" t="s">
-        <v>1334</v>
+        <v>1318</v>
       </c>
     </row>
     <row r="329" spans="1:7" x14ac:dyDescent="0.3">
@@ -12197,10 +12197,10 @@
         <v>603</v>
       </c>
       <c r="F329" s="11" t="s">
-        <v>1335</v>
+        <v>1319</v>
       </c>
       <c r="G329" s="11" t="s">
-        <v>1336</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="330" spans="1:7" x14ac:dyDescent="0.3">
@@ -12220,10 +12220,10 @@
         <v>603</v>
       </c>
       <c r="F330" s="11" t="s">
-        <v>1337</v>
+        <v>1321</v>
       </c>
       <c r="G330" s="11" t="s">
-        <v>1338</v>
+        <v>1322</v>
       </c>
     </row>
     <row r="331" spans="1:7" x14ac:dyDescent="0.3">
@@ -12243,10 +12243,10 @@
         <v>603</v>
       </c>
       <c r="F331" s="11" t="s">
-        <v>1339</v>
+        <v>1323</v>
       </c>
       <c r="G331" s="11" t="s">
-        <v>1340</v>
+        <v>1324</v>
       </c>
     </row>
     <row r="332" spans="1:7" x14ac:dyDescent="0.3">
@@ -12266,10 +12266,10 @@
         <v>603</v>
       </c>
       <c r="F332" s="11" t="s">
-        <v>1341</v>
+        <v>1325</v>
       </c>
       <c r="G332" s="11" t="s">
-        <v>1342</v>
+        <v>1326</v>
       </c>
     </row>
     <row r="333" spans="1:7" x14ac:dyDescent="0.3">
@@ -12289,10 +12289,10 @@
         <v>603</v>
       </c>
       <c r="F333" s="11" t="s">
-        <v>1343</v>
+        <v>1327</v>
       </c>
       <c r="G333" s="11" t="s">
-        <v>1344</v>
+        <v>1328</v>
       </c>
     </row>
     <row r="334" spans="1:7" x14ac:dyDescent="0.3">
@@ -12312,10 +12312,10 @@
         <v>603</v>
       </c>
       <c r="F334" s="11" t="s">
-        <v>1345</v>
+        <v>1329</v>
       </c>
       <c r="G334" s="11" t="s">
-        <v>1346</v>
+        <v>1330</v>
       </c>
     </row>
     <row r="335" spans="1:7" x14ac:dyDescent="0.3">
@@ -12335,10 +12335,10 @@
         <v>603</v>
       </c>
       <c r="F335" s="11" t="s">
-        <v>1347</v>
+        <v>1331</v>
       </c>
       <c r="G335" s="11" t="s">
-        <v>1348</v>
+        <v>1332</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Adhiparasakthi Students Data 1.xlsx
</commit_message>
<xml_diff>
--- a/files/Adhiparasakthi Students Data 1.xlsx
+++ b/files/Adhiparasakthi Students Data 1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vigne\Google_Backup\Github\sb4c\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E42DE63E-E73B-423E-9195-E867206429ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD490F28-3535-4073-904A-E89555E29F50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E3F0EEA9-6BAE-46A1-95E3-E9CE509FC50B}"/>
   </bookViews>
@@ -2625,12 +2625,6 @@
     <t>Edu#970864</t>
   </si>
   <si>
-    <t>EFIBM26927896787@edunetmail.com</t>
-  </si>
-  <si>
-    <t>Edu#666852</t>
-  </si>
-  <si>
     <t>EFIBM26220428119@edunetmail.com</t>
   </si>
   <si>
@@ -4084,6 +4078,12 @@
   </si>
   <si>
     <t>Edu#495569</t>
+  </si>
+  <si>
+    <t>EFIBM26239586755@edunetmail.com</t>
+  </si>
+  <si>
+    <t>Edu#289354</t>
   </si>
 </sst>
 </file>
@@ -6257,10 +6257,10 @@
         <v>138</v>
       </c>
       <c r="F68" s="12" t="s">
-        <v>1301</v>
+        <v>1299</v>
       </c>
       <c r="G68" s="12" t="s">
-        <v>1302</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="69" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -6294,7 +6294,7 @@
         <v>141</v>
       </c>
       <c r="C70" s="16" t="s">
-        <v>1337</v>
+        <v>1335</v>
       </c>
       <c r="D70" s="1" t="s">
         <v>188</v>
@@ -6303,10 +6303,10 @@
         <v>138</v>
       </c>
       <c r="F70" s="12" t="s">
-        <v>1335</v>
+        <v>1333</v>
       </c>
       <c r="G70" s="12" t="s">
-        <v>1336</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="71" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -6510,10 +6510,10 @@
         <v>138</v>
       </c>
       <c r="F79" s="12" t="s">
-        <v>1333</v>
+        <v>1331</v>
       </c>
       <c r="G79" s="12" t="s">
-        <v>1334</v>
+        <v>1332</v>
       </c>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.3">
@@ -6556,10 +6556,10 @@
         <v>138</v>
       </c>
       <c r="F81" s="11" t="s">
-        <v>1325</v>
+        <v>1323</v>
       </c>
       <c r="G81" s="11" t="s">
-        <v>1326</v>
+        <v>1324</v>
       </c>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.3">
@@ -6625,10 +6625,10 @@
         <v>138</v>
       </c>
       <c r="F84" s="11" t="s">
-        <v>1315</v>
+        <v>1313</v>
       </c>
       <c r="G84" s="11" t="s">
-        <v>1316</v>
+        <v>1314</v>
       </c>
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.3">
@@ -6648,10 +6648,10 @@
         <v>138</v>
       </c>
       <c r="F85" s="11" t="s">
-        <v>1327</v>
+        <v>1325</v>
       </c>
       <c r="G85" s="11" t="s">
-        <v>1328</v>
+        <v>1326</v>
       </c>
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.3">
@@ -6763,10 +6763,10 @@
         <v>138</v>
       </c>
       <c r="F90" s="11" t="s">
-        <v>1317</v>
+        <v>1315</v>
       </c>
       <c r="G90" s="11" t="s">
-        <v>1318</v>
+        <v>1316</v>
       </c>
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.3">
@@ -6992,11 +6992,11 @@
       <c r="E100" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="F100" s="6" t="s">
-        <v>863</v>
-      </c>
-      <c r="G100" s="8" t="s">
-        <v>864</v>
+      <c r="F100" s="5" t="s">
+        <v>1348</v>
+      </c>
+      <c r="G100" s="7" t="s">
+        <v>1349</v>
       </c>
     </row>
     <row r="101" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7016,10 +7016,10 @@
         <v>138</v>
       </c>
       <c r="F101" s="6" t="s">
-        <v>865</v>
+        <v>863</v>
       </c>
       <c r="G101" s="8" t="s">
-        <v>866</v>
+        <v>864</v>
       </c>
     </row>
     <row r="102" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7039,10 +7039,10 @@
         <v>138</v>
       </c>
       <c r="F102" s="6" t="s">
-        <v>867</v>
+        <v>865</v>
       </c>
       <c r="G102" s="8" t="s">
-        <v>868</v>
+        <v>866</v>
       </c>
     </row>
     <row r="103" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7062,10 +7062,10 @@
         <v>138</v>
       </c>
       <c r="F103" s="6" t="s">
-        <v>869</v>
+        <v>867</v>
       </c>
       <c r="G103" s="8" t="s">
-        <v>870</v>
+        <v>868</v>
       </c>
     </row>
     <row r="104" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7085,10 +7085,10 @@
         <v>138</v>
       </c>
       <c r="F104" s="6" t="s">
-        <v>871</v>
+        <v>869</v>
       </c>
       <c r="G104" s="8" t="s">
-        <v>872</v>
+        <v>870</v>
       </c>
     </row>
     <row r="105" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7108,10 +7108,10 @@
         <v>138</v>
       </c>
       <c r="F105" s="12" t="s">
-        <v>1340</v>
+        <v>1338</v>
       </c>
       <c r="G105" s="12" t="s">
-        <v>1341</v>
+        <v>1339</v>
       </c>
     </row>
     <row r="106" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7131,10 +7131,10 @@
         <v>138</v>
       </c>
       <c r="F106" s="6" t="s">
-        <v>873</v>
+        <v>871</v>
       </c>
       <c r="G106" s="8" t="s">
-        <v>874</v>
+        <v>872</v>
       </c>
     </row>
     <row r="107" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7154,10 +7154,10 @@
         <v>138</v>
       </c>
       <c r="F107" s="5" t="s">
-        <v>1348</v>
+        <v>1346</v>
       </c>
       <c r="G107" s="7" t="s">
-        <v>1349</v>
+        <v>1347</v>
       </c>
     </row>
     <row r="108" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7177,10 +7177,10 @@
         <v>138</v>
       </c>
       <c r="F108" s="6" t="s">
-        <v>875</v>
+        <v>873</v>
       </c>
       <c r="G108" s="8" t="s">
-        <v>876</v>
+        <v>874</v>
       </c>
     </row>
     <row r="109" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7200,10 +7200,10 @@
         <v>138</v>
       </c>
       <c r="F109" s="6" t="s">
-        <v>877</v>
+        <v>875</v>
       </c>
       <c r="G109" s="8" t="s">
-        <v>878</v>
+        <v>876</v>
       </c>
     </row>
     <row r="110" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7223,10 +7223,10 @@
         <v>138</v>
       </c>
       <c r="F110" s="6" t="s">
-        <v>879</v>
+        <v>877</v>
       </c>
       <c r="G110" s="8" t="s">
-        <v>880</v>
+        <v>878</v>
       </c>
     </row>
     <row r="111" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7246,10 +7246,10 @@
         <v>138</v>
       </c>
       <c r="F111" s="6" t="s">
-        <v>881</v>
+        <v>879</v>
       </c>
       <c r="G111" s="8" t="s">
-        <v>882</v>
+        <v>880</v>
       </c>
     </row>
     <row r="112" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7269,10 +7269,10 @@
         <v>138</v>
       </c>
       <c r="F112" s="17" t="s">
-        <v>1346</v>
+        <v>1344</v>
       </c>
       <c r="G112" s="17" t="s">
-        <v>1347</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="113" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7292,10 +7292,10 @@
         <v>138</v>
       </c>
       <c r="F113" s="6" t="s">
-        <v>883</v>
+        <v>881</v>
       </c>
       <c r="G113" s="8" t="s">
-        <v>884</v>
+        <v>882</v>
       </c>
     </row>
     <row r="114" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7315,10 +7315,10 @@
         <v>138</v>
       </c>
       <c r="F114" s="12" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="G114" s="12" t="s">
-        <v>1343</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="115" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7338,10 +7338,10 @@
         <v>138</v>
       </c>
       <c r="F115" s="6" t="s">
-        <v>885</v>
+        <v>883</v>
       </c>
       <c r="G115" s="8" t="s">
-        <v>886</v>
+        <v>884</v>
       </c>
     </row>
     <row r="116" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7361,10 +7361,10 @@
         <v>138</v>
       </c>
       <c r="F116" s="6" t="s">
-        <v>887</v>
+        <v>885</v>
       </c>
       <c r="G116" s="8" t="s">
-        <v>888</v>
+        <v>886</v>
       </c>
     </row>
     <row r="117" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7384,10 +7384,10 @@
         <v>138</v>
       </c>
       <c r="F117" s="6" t="s">
-        <v>889</v>
+        <v>887</v>
       </c>
       <c r="G117" s="8" t="s">
-        <v>890</v>
+        <v>888</v>
       </c>
     </row>
     <row r="118" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7404,10 +7404,10 @@
         <v>138</v>
       </c>
       <c r="F118" s="6" t="s">
-        <v>891</v>
+        <v>889</v>
       </c>
       <c r="G118" s="8" t="s">
-        <v>892</v>
+        <v>890</v>
       </c>
     </row>
     <row r="119" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7427,10 +7427,10 @@
         <v>138</v>
       </c>
       <c r="F119" s="12" t="s">
-        <v>1338</v>
+        <v>1336</v>
       </c>
       <c r="G119" s="12" t="s">
-        <v>1339</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="120" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7450,10 +7450,10 @@
         <v>138</v>
       </c>
       <c r="F120" s="6" t="s">
-        <v>893</v>
+        <v>891</v>
       </c>
       <c r="G120" s="8" t="s">
-        <v>894</v>
+        <v>892</v>
       </c>
     </row>
     <row r="121" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7473,10 +7473,10 @@
         <v>138</v>
       </c>
       <c r="F121" s="12" t="s">
-        <v>1344</v>
+        <v>1342</v>
       </c>
       <c r="G121" s="12" t="s">
-        <v>1345</v>
+        <v>1343</v>
       </c>
     </row>
     <row r="122" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7496,10 +7496,10 @@
         <v>138</v>
       </c>
       <c r="F122" s="6" t="s">
-        <v>895</v>
+        <v>893</v>
       </c>
       <c r="G122" s="8" t="s">
-        <v>896</v>
+        <v>894</v>
       </c>
     </row>
     <row r="123" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7519,10 +7519,10 @@
         <v>138</v>
       </c>
       <c r="F123" s="6" t="s">
-        <v>897</v>
+        <v>895</v>
       </c>
       <c r="G123" s="8" t="s">
-        <v>898</v>
+        <v>896</v>
       </c>
     </row>
     <row r="124" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7542,10 +7542,10 @@
         <v>138</v>
       </c>
       <c r="F124" s="6" t="s">
-        <v>899</v>
+        <v>897</v>
       </c>
       <c r="G124" s="8" t="s">
-        <v>900</v>
+        <v>898</v>
       </c>
     </row>
     <row r="125" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7565,10 +7565,10 @@
         <v>138</v>
       </c>
       <c r="F125" s="12" t="s">
-        <v>1307</v>
+        <v>1305</v>
       </c>
       <c r="G125" s="12" t="s">
-        <v>1308</v>
+        <v>1306</v>
       </c>
     </row>
     <row r="126" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7588,10 +7588,10 @@
         <v>138</v>
       </c>
       <c r="F126" s="12" t="s">
-        <v>1321</v>
+        <v>1319</v>
       </c>
       <c r="G126" s="12" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="127" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7611,10 +7611,10 @@
         <v>138</v>
       </c>
       <c r="F127" s="6" t="s">
-        <v>901</v>
+        <v>899</v>
       </c>
       <c r="G127" s="8" t="s">
-        <v>902</v>
+        <v>900</v>
       </c>
     </row>
     <row r="128" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7634,10 +7634,10 @@
         <v>138</v>
       </c>
       <c r="F128" s="6" t="s">
-        <v>903</v>
+        <v>901</v>
       </c>
       <c r="G128" s="8" t="s">
-        <v>904</v>
+        <v>902</v>
       </c>
     </row>
     <row r="129" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7657,10 +7657,10 @@
         <v>138</v>
       </c>
       <c r="F129" s="6" t="s">
-        <v>905</v>
+        <v>903</v>
       </c>
       <c r="G129" s="8" t="s">
-        <v>906</v>
+        <v>904</v>
       </c>
     </row>
     <row r="130" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7680,10 +7680,10 @@
         <v>138</v>
       </c>
       <c r="F130" s="12" t="s">
-        <v>1329</v>
+        <v>1327</v>
       </c>
       <c r="G130" s="12" t="s">
-        <v>1330</v>
+        <v>1328</v>
       </c>
     </row>
     <row r="131" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7703,10 +7703,10 @@
         <v>138</v>
       </c>
       <c r="F131" s="6" t="s">
-        <v>907</v>
+        <v>905</v>
       </c>
       <c r="G131" s="8" t="s">
-        <v>908</v>
+        <v>906</v>
       </c>
     </row>
     <row r="132" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7726,10 +7726,10 @@
         <v>138</v>
       </c>
       <c r="F132" s="6" t="s">
-        <v>909</v>
+        <v>907</v>
       </c>
       <c r="G132" s="8" t="s">
-        <v>910</v>
+        <v>908</v>
       </c>
     </row>
     <row r="133" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7749,10 +7749,10 @@
         <v>138</v>
       </c>
       <c r="F133" s="6" t="s">
-        <v>911</v>
+        <v>909</v>
       </c>
       <c r="G133" s="8" t="s">
-        <v>912</v>
+        <v>910</v>
       </c>
     </row>
     <row r="134" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7772,10 +7772,10 @@
         <v>138</v>
       </c>
       <c r="F134" s="6" t="s">
-        <v>913</v>
+        <v>911</v>
       </c>
       <c r="G134" s="8" t="s">
-        <v>914</v>
+        <v>912</v>
       </c>
     </row>
     <row r="135" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7795,10 +7795,10 @@
         <v>138</v>
       </c>
       <c r="F135" s="12" t="s">
-        <v>1313</v>
+        <v>1311</v>
       </c>
       <c r="G135" s="12" t="s">
-        <v>1314</v>
+        <v>1312</v>
       </c>
     </row>
     <row r="136" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7818,10 +7818,10 @@
         <v>138</v>
       </c>
       <c r="F136" s="6" t="s">
-        <v>915</v>
+        <v>913</v>
       </c>
       <c r="G136" s="8" t="s">
-        <v>916</v>
+        <v>914</v>
       </c>
     </row>
     <row r="137" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7841,10 +7841,10 @@
         <v>138</v>
       </c>
       <c r="F137" s="6" t="s">
-        <v>917</v>
+        <v>915</v>
       </c>
       <c r="G137" s="8" t="s">
-        <v>918</v>
+        <v>916</v>
       </c>
     </row>
     <row r="138" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7864,10 +7864,10 @@
         <v>138</v>
       </c>
       <c r="F138" s="6" t="s">
-        <v>919</v>
+        <v>917</v>
       </c>
       <c r="G138" s="8" t="s">
-        <v>920</v>
+        <v>918</v>
       </c>
     </row>
     <row r="139" spans="1:7" x14ac:dyDescent="0.3">
@@ -7887,10 +7887,10 @@
         <v>138</v>
       </c>
       <c r="F139" s="9" t="s">
-        <v>921</v>
+        <v>919</v>
       </c>
       <c r="G139" s="10" t="s">
-        <v>922</v>
+        <v>920</v>
       </c>
     </row>
     <row r="140" spans="1:7" x14ac:dyDescent="0.3">
@@ -7910,10 +7910,10 @@
         <v>138</v>
       </c>
       <c r="F140" s="15" t="s">
-        <v>923</v>
+        <v>921</v>
       </c>
       <c r="G140" s="15" t="s">
-        <v>924</v>
+        <v>922</v>
       </c>
     </row>
     <row r="141" spans="1:7" x14ac:dyDescent="0.3">
@@ -7933,10 +7933,10 @@
         <v>138</v>
       </c>
       <c r="F141" s="11" t="s">
-        <v>1303</v>
+        <v>1301</v>
       </c>
       <c r="G141" s="11" t="s">
-        <v>1304</v>
+        <v>1302</v>
       </c>
     </row>
     <row r="142" spans="1:7" x14ac:dyDescent="0.3">
@@ -7956,10 +7956,10 @@
         <v>138</v>
       </c>
       <c r="F142" s="15" t="s">
-        <v>925</v>
+        <v>923</v>
       </c>
       <c r="G142" s="15" t="s">
-        <v>926</v>
+        <v>924</v>
       </c>
     </row>
     <row r="143" spans="1:7" x14ac:dyDescent="0.3">
@@ -7979,10 +7979,10 @@
         <v>138</v>
       </c>
       <c r="F143" s="11" t="s">
-        <v>1331</v>
+        <v>1329</v>
       </c>
       <c r="G143" s="11" t="s">
-        <v>1332</v>
+        <v>1330</v>
       </c>
     </row>
     <row r="144" spans="1:7" x14ac:dyDescent="0.3">
@@ -8002,10 +8002,10 @@
         <v>138</v>
       </c>
       <c r="F144" s="11" t="s">
-        <v>1305</v>
+        <v>1303</v>
       </c>
       <c r="G144" s="11" t="s">
-        <v>1306</v>
+        <v>1304</v>
       </c>
     </row>
     <row r="145" spans="1:7" x14ac:dyDescent="0.3">
@@ -8025,10 +8025,10 @@
         <v>138</v>
       </c>
       <c r="F145" s="15" t="s">
-        <v>927</v>
+        <v>925</v>
       </c>
       <c r="G145" s="15" t="s">
-        <v>928</v>
+        <v>926</v>
       </c>
     </row>
     <row r="146" spans="1:7" x14ac:dyDescent="0.3">
@@ -8048,10 +8048,10 @@
         <v>138</v>
       </c>
       <c r="F146" s="11" t="s">
-        <v>1311</v>
+        <v>1309</v>
       </c>
       <c r="G146" s="11" t="s">
-        <v>1312</v>
+        <v>1310</v>
       </c>
     </row>
     <row r="147" spans="1:7" x14ac:dyDescent="0.3">
@@ -8071,10 +8071,10 @@
         <v>138</v>
       </c>
       <c r="F147" s="15" t="s">
-        <v>929</v>
+        <v>927</v>
       </c>
       <c r="G147" s="15" t="s">
-        <v>930</v>
+        <v>928</v>
       </c>
     </row>
     <row r="148" spans="1:7" x14ac:dyDescent="0.3">
@@ -8094,10 +8094,10 @@
         <v>138</v>
       </c>
       <c r="F148" s="15" t="s">
-        <v>931</v>
+        <v>929</v>
       </c>
       <c r="G148" s="15" t="s">
-        <v>932</v>
+        <v>930</v>
       </c>
     </row>
     <row r="149" spans="1:7" x14ac:dyDescent="0.3">
@@ -8117,10 +8117,10 @@
         <v>138</v>
       </c>
       <c r="F149" s="15" t="s">
-        <v>933</v>
+        <v>931</v>
       </c>
       <c r="G149" s="15" t="s">
-        <v>934</v>
+        <v>932</v>
       </c>
     </row>
     <row r="150" spans="1:7" x14ac:dyDescent="0.3">
@@ -8140,10 +8140,10 @@
         <v>138</v>
       </c>
       <c r="F150" s="15" t="s">
-        <v>935</v>
+        <v>933</v>
       </c>
       <c r="G150" s="15" t="s">
-        <v>936</v>
+        <v>934</v>
       </c>
     </row>
     <row r="151" spans="1:7" x14ac:dyDescent="0.3">
@@ -8163,10 +8163,10 @@
         <v>138</v>
       </c>
       <c r="F151" s="15" t="s">
-        <v>937</v>
+        <v>935</v>
       </c>
       <c r="G151" s="15" t="s">
-        <v>938</v>
+        <v>936</v>
       </c>
     </row>
     <row r="152" spans="1:7" x14ac:dyDescent="0.3">
@@ -8186,10 +8186,10 @@
         <v>138</v>
       </c>
       <c r="F152" s="11" t="s">
-        <v>1319</v>
+        <v>1317</v>
       </c>
       <c r="G152" s="11" t="s">
-        <v>1320</v>
+        <v>1318</v>
       </c>
     </row>
     <row r="153" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8209,10 +8209,10 @@
         <v>138</v>
       </c>
       <c r="F153" s="13" t="s">
-        <v>939</v>
+        <v>937</v>
       </c>
       <c r="G153" s="14" t="s">
-        <v>940</v>
+        <v>938</v>
       </c>
     </row>
     <row r="154" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8232,10 +8232,10 @@
         <v>138</v>
       </c>
       <c r="F154" s="6" t="s">
-        <v>941</v>
+        <v>939</v>
       </c>
       <c r="G154" s="8" t="s">
-        <v>942</v>
+        <v>940</v>
       </c>
     </row>
     <row r="155" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8255,10 +8255,10 @@
         <v>138</v>
       </c>
       <c r="F155" s="6" t="s">
-        <v>943</v>
+        <v>941</v>
       </c>
       <c r="G155" s="8" t="s">
-        <v>944</v>
+        <v>942</v>
       </c>
     </row>
     <row r="156" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8278,10 +8278,10 @@
         <v>138</v>
       </c>
       <c r="F156" s="6" t="s">
-        <v>945</v>
+        <v>943</v>
       </c>
       <c r="G156" s="8" t="s">
-        <v>946</v>
+        <v>944</v>
       </c>
     </row>
     <row r="157" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8301,10 +8301,10 @@
         <v>138</v>
       </c>
       <c r="F157" s="12" t="s">
-        <v>1323</v>
+        <v>1321</v>
       </c>
       <c r="G157" s="12" t="s">
-        <v>1324</v>
+        <v>1322</v>
       </c>
     </row>
     <row r="158" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8324,10 +8324,10 @@
         <v>138</v>
       </c>
       <c r="F158" s="6" t="s">
-        <v>947</v>
+        <v>945</v>
       </c>
       <c r="G158" s="8" t="s">
-        <v>948</v>
+        <v>946</v>
       </c>
     </row>
     <row r="159" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8347,10 +8347,10 @@
         <v>138</v>
       </c>
       <c r="F159" s="6" t="s">
-        <v>949</v>
+        <v>947</v>
       </c>
       <c r="G159" s="8" t="s">
-        <v>950</v>
+        <v>948</v>
       </c>
     </row>
     <row r="160" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8370,10 +8370,10 @@
         <v>138</v>
       </c>
       <c r="F160" s="12" t="s">
-        <v>1309</v>
+        <v>1307</v>
       </c>
       <c r="G160" s="12" t="s">
-        <v>1310</v>
+        <v>1308</v>
       </c>
     </row>
     <row r="161" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8393,10 +8393,10 @@
         <v>138</v>
       </c>
       <c r="F161" s="6" t="s">
-        <v>951</v>
+        <v>949</v>
       </c>
       <c r="G161" s="8" t="s">
-        <v>952</v>
+        <v>950</v>
       </c>
     </row>
     <row r="162" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8416,10 +8416,10 @@
         <v>138</v>
       </c>
       <c r="F162" s="6" t="s">
-        <v>953</v>
+        <v>951</v>
       </c>
       <c r="G162" s="8" t="s">
-        <v>954</v>
+        <v>952</v>
       </c>
     </row>
     <row r="163" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8439,10 +8439,10 @@
         <v>138</v>
       </c>
       <c r="F163" s="6" t="s">
-        <v>955</v>
+        <v>953</v>
       </c>
       <c r="G163" s="8" t="s">
-        <v>956</v>
+        <v>954</v>
       </c>
     </row>
     <row r="164" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8462,10 +8462,10 @@
         <v>138</v>
       </c>
       <c r="F164" s="6" t="s">
-        <v>957</v>
+        <v>955</v>
       </c>
       <c r="G164" s="8" t="s">
-        <v>958</v>
+        <v>956</v>
       </c>
     </row>
     <row r="165" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8485,10 +8485,10 @@
         <v>138</v>
       </c>
       <c r="F165" s="6" t="s">
-        <v>959</v>
+        <v>957</v>
       </c>
       <c r="G165" s="8" t="s">
-        <v>960</v>
+        <v>958</v>
       </c>
     </row>
     <row r="166" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8508,10 +8508,10 @@
         <v>138</v>
       </c>
       <c r="F166" s="6" t="s">
-        <v>961</v>
+        <v>959</v>
       </c>
       <c r="G166" s="8" t="s">
-        <v>962</v>
+        <v>960</v>
       </c>
     </row>
     <row r="167" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8531,10 +8531,10 @@
         <v>138</v>
       </c>
       <c r="F167" s="6" t="s">
-        <v>963</v>
+        <v>961</v>
       </c>
       <c r="G167" s="8" t="s">
-        <v>964</v>
+        <v>962</v>
       </c>
     </row>
     <row r="168" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8554,10 +8554,10 @@
         <v>138</v>
       </c>
       <c r="F168" s="6" t="s">
-        <v>965</v>
+        <v>963</v>
       </c>
       <c r="G168" s="8" t="s">
-        <v>966</v>
+        <v>964</v>
       </c>
     </row>
     <row r="169" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8577,10 +8577,10 @@
         <v>138</v>
       </c>
       <c r="F169" s="6" t="s">
-        <v>967</v>
+        <v>965</v>
       </c>
       <c r="G169" s="8" t="s">
-        <v>968</v>
+        <v>966</v>
       </c>
     </row>
     <row r="170" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8600,10 +8600,10 @@
         <v>138</v>
       </c>
       <c r="F170" s="6" t="s">
-        <v>969</v>
+        <v>967</v>
       </c>
       <c r="G170" s="8" t="s">
-        <v>970</v>
+        <v>968</v>
       </c>
     </row>
     <row r="171" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8623,10 +8623,10 @@
         <v>138</v>
       </c>
       <c r="F171" s="6" t="s">
-        <v>971</v>
+        <v>969</v>
       </c>
       <c r="G171" s="8" t="s">
-        <v>972</v>
+        <v>970</v>
       </c>
     </row>
     <row r="172" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8646,10 +8646,10 @@
         <v>138</v>
       </c>
       <c r="F172" s="6" t="s">
-        <v>973</v>
+        <v>971</v>
       </c>
       <c r="G172" s="8" t="s">
-        <v>974</v>
+        <v>972</v>
       </c>
     </row>
     <row r="173" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8669,10 +8669,10 @@
         <v>138</v>
       </c>
       <c r="F173" s="6" t="s">
-        <v>975</v>
+        <v>973</v>
       </c>
       <c r="G173" s="8" t="s">
-        <v>976</v>
+        <v>974</v>
       </c>
     </row>
     <row r="174" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8692,10 +8692,10 @@
         <v>138</v>
       </c>
       <c r="F174" s="6" t="s">
-        <v>977</v>
+        <v>975</v>
       </c>
       <c r="G174" s="8" t="s">
-        <v>978</v>
+        <v>976</v>
       </c>
     </row>
     <row r="175" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8715,10 +8715,10 @@
         <v>138</v>
       </c>
       <c r="F175" s="6" t="s">
-        <v>979</v>
+        <v>977</v>
       </c>
       <c r="G175" s="8" t="s">
-        <v>980</v>
+        <v>978</v>
       </c>
     </row>
     <row r="176" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8738,10 +8738,10 @@
         <v>138</v>
       </c>
       <c r="F176" s="6" t="s">
-        <v>981</v>
+        <v>979</v>
       </c>
       <c r="G176" s="8" t="s">
-        <v>982</v>
+        <v>980</v>
       </c>
     </row>
     <row r="177" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8761,10 +8761,10 @@
         <v>138</v>
       </c>
       <c r="F177" s="6" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="G177" s="8" t="s">
-        <v>984</v>
+        <v>982</v>
       </c>
     </row>
     <row r="178" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8784,10 +8784,10 @@
         <v>138</v>
       </c>
       <c r="F178" s="6" t="s">
-        <v>985</v>
+        <v>983</v>
       </c>
       <c r="G178" s="8" t="s">
-        <v>986</v>
+        <v>984</v>
       </c>
     </row>
     <row r="179" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8807,10 +8807,10 @@
         <v>138</v>
       </c>
       <c r="F179" s="6" t="s">
-        <v>987</v>
+        <v>985</v>
       </c>
       <c r="G179" s="8" t="s">
-        <v>988</v>
+        <v>986</v>
       </c>
     </row>
     <row r="180" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8830,10 +8830,10 @@
         <v>138</v>
       </c>
       <c r="F180" s="6" t="s">
-        <v>989</v>
+        <v>987</v>
       </c>
       <c r="G180" s="8" t="s">
-        <v>990</v>
+        <v>988</v>
       </c>
     </row>
     <row r="181" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8853,10 +8853,10 @@
         <v>138</v>
       </c>
       <c r="F181" s="6" t="s">
-        <v>991</v>
+        <v>989</v>
       </c>
       <c r="G181" s="8" t="s">
-        <v>992</v>
+        <v>990</v>
       </c>
     </row>
     <row r="182" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8876,10 +8876,10 @@
         <v>138</v>
       </c>
       <c r="F182" s="6" t="s">
-        <v>993</v>
+        <v>991</v>
       </c>
       <c r="G182" s="8" t="s">
-        <v>994</v>
+        <v>992</v>
       </c>
     </row>
     <row r="183" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8899,10 +8899,10 @@
         <v>138</v>
       </c>
       <c r="F183" s="6" t="s">
-        <v>995</v>
+        <v>993</v>
       </c>
       <c r="G183" s="8" t="s">
-        <v>996</v>
+        <v>994</v>
       </c>
     </row>
     <row r="184" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8922,10 +8922,10 @@
         <v>138</v>
       </c>
       <c r="F184" s="6" t="s">
-        <v>997</v>
+        <v>995</v>
       </c>
       <c r="G184" s="8" t="s">
-        <v>998</v>
+        <v>996</v>
       </c>
     </row>
     <row r="185" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8945,10 +8945,10 @@
         <v>138</v>
       </c>
       <c r="F185" s="6" t="s">
-        <v>999</v>
+        <v>997</v>
       </c>
       <c r="G185" s="8" t="s">
-        <v>1000</v>
+        <v>998</v>
       </c>
     </row>
     <row r="186" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8968,10 +8968,10 @@
         <v>138</v>
       </c>
       <c r="F186" s="6" t="s">
-        <v>1001</v>
+        <v>999</v>
       </c>
       <c r="G186" s="8" t="s">
-        <v>1002</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="187" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -8991,10 +8991,10 @@
         <v>138</v>
       </c>
       <c r="F187" s="6" t="s">
-        <v>1003</v>
+        <v>1001</v>
       </c>
       <c r="G187" s="8" t="s">
-        <v>1004</v>
+        <v>1002</v>
       </c>
     </row>
     <row r="188" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9014,10 +9014,10 @@
         <v>138</v>
       </c>
       <c r="F188" s="6" t="s">
-        <v>1005</v>
+        <v>1003</v>
       </c>
       <c r="G188" s="8" t="s">
-        <v>1006</v>
+        <v>1004</v>
       </c>
     </row>
     <row r="189" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9037,10 +9037,10 @@
         <v>138</v>
       </c>
       <c r="F189" s="6" t="s">
-        <v>1007</v>
+        <v>1005</v>
       </c>
       <c r="G189" s="8" t="s">
-        <v>1008</v>
+        <v>1006</v>
       </c>
     </row>
     <row r="190" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9060,10 +9060,10 @@
         <v>138</v>
       </c>
       <c r="F190" s="6" t="s">
-        <v>1009</v>
+        <v>1007</v>
       </c>
       <c r="G190" s="8" t="s">
-        <v>1010</v>
+        <v>1008</v>
       </c>
     </row>
     <row r="191" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9083,10 +9083,10 @@
         <v>138</v>
       </c>
       <c r="F191" s="6" t="s">
-        <v>1011</v>
+        <v>1009</v>
       </c>
       <c r="G191" s="8" t="s">
-        <v>1012</v>
+        <v>1010</v>
       </c>
     </row>
     <row r="192" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9106,10 +9106,10 @@
         <v>138</v>
       </c>
       <c r="F192" s="6" t="s">
-        <v>1013</v>
+        <v>1011</v>
       </c>
       <c r="G192" s="8" t="s">
-        <v>1014</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="193" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9129,10 +9129,10 @@
         <v>138</v>
       </c>
       <c r="F193" s="6" t="s">
-        <v>1015</v>
+        <v>1013</v>
       </c>
       <c r="G193" s="8" t="s">
-        <v>1016</v>
+        <v>1014</v>
       </c>
     </row>
     <row r="194" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9152,10 +9152,10 @@
         <v>138</v>
       </c>
       <c r="F194" s="6" t="s">
-        <v>1017</v>
+        <v>1015</v>
       </c>
       <c r="G194" s="8" t="s">
-        <v>1018</v>
+        <v>1016</v>
       </c>
     </row>
     <row r="195" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9175,10 +9175,10 @@
         <v>138</v>
       </c>
       <c r="F195" s="6" t="s">
-        <v>1019</v>
+        <v>1017</v>
       </c>
       <c r="G195" s="8" t="s">
-        <v>1020</v>
+        <v>1018</v>
       </c>
     </row>
     <row r="196" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9198,10 +9198,10 @@
         <v>138</v>
       </c>
       <c r="F196" s="6" t="s">
-        <v>1021</v>
+        <v>1019</v>
       </c>
       <c r="G196" s="8" t="s">
-        <v>1022</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="197" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9221,10 +9221,10 @@
         <v>138</v>
       </c>
       <c r="F197" s="6" t="s">
-        <v>1023</v>
+        <v>1021</v>
       </c>
       <c r="G197" s="8" t="s">
-        <v>1024</v>
+        <v>1022</v>
       </c>
     </row>
     <row r="198" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9244,10 +9244,10 @@
         <v>138</v>
       </c>
       <c r="F198" s="6" t="s">
-        <v>1025</v>
+        <v>1023</v>
       </c>
       <c r="G198" s="8" t="s">
-        <v>1026</v>
+        <v>1024</v>
       </c>
     </row>
     <row r="199" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9267,10 +9267,10 @@
         <v>138</v>
       </c>
       <c r="F199" s="6" t="s">
-        <v>1027</v>
+        <v>1025</v>
       </c>
       <c r="G199" s="8" t="s">
-        <v>1028</v>
+        <v>1026</v>
       </c>
     </row>
     <row r="200" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9290,10 +9290,10 @@
         <v>138</v>
       </c>
       <c r="F200" s="6" t="s">
-        <v>1029</v>
+        <v>1027</v>
       </c>
       <c r="G200" s="8" t="s">
-        <v>1030</v>
+        <v>1028</v>
       </c>
     </row>
     <row r="201" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9313,10 +9313,10 @@
         <v>138</v>
       </c>
       <c r="F201" s="6" t="s">
-        <v>1031</v>
+        <v>1029</v>
       </c>
       <c r="G201" s="8" t="s">
-        <v>1032</v>
+        <v>1030</v>
       </c>
     </row>
     <row r="202" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9336,10 +9336,10 @@
         <v>138</v>
       </c>
       <c r="F202" s="6" t="s">
-        <v>1033</v>
+        <v>1031</v>
       </c>
       <c r="G202" s="8" t="s">
-        <v>1034</v>
+        <v>1032</v>
       </c>
     </row>
     <row r="203" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9359,10 +9359,10 @@
         <v>138</v>
       </c>
       <c r="F203" s="6" t="s">
-        <v>1035</v>
+        <v>1033</v>
       </c>
       <c r="G203" s="8" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
     </row>
     <row r="204" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9382,10 +9382,10 @@
         <v>138</v>
       </c>
       <c r="F204" s="6" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
       <c r="G204" s="8" t="s">
-        <v>1038</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="205" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9405,10 +9405,10 @@
         <v>138</v>
       </c>
       <c r="F205" s="6" t="s">
-        <v>1039</v>
+        <v>1037</v>
       </c>
       <c r="G205" s="8" t="s">
-        <v>1040</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="206" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9428,10 +9428,10 @@
         <v>138</v>
       </c>
       <c r="F206" s="6" t="s">
-        <v>1041</v>
+        <v>1039</v>
       </c>
       <c r="G206" s="8" t="s">
-        <v>1042</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="207" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9451,10 +9451,10 @@
         <v>138</v>
       </c>
       <c r="F207" s="6" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
       <c r="G207" s="8" t="s">
-        <v>1044</v>
+        <v>1042</v>
       </c>
     </row>
     <row r="208" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9474,10 +9474,10 @@
         <v>138</v>
       </c>
       <c r="F208" s="6" t="s">
-        <v>1045</v>
+        <v>1043</v>
       </c>
       <c r="G208" s="8" t="s">
-        <v>1046</v>
+        <v>1044</v>
       </c>
     </row>
     <row r="209" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9497,10 +9497,10 @@
         <v>138</v>
       </c>
       <c r="F209" s="6" t="s">
-        <v>1047</v>
+        <v>1045</v>
       </c>
       <c r="G209" s="8" t="s">
-        <v>1048</v>
+        <v>1046</v>
       </c>
     </row>
     <row r="210" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9520,10 +9520,10 @@
         <v>138</v>
       </c>
       <c r="F210" s="6" t="s">
-        <v>1049</v>
+        <v>1047</v>
       </c>
       <c r="G210" s="8" t="s">
-        <v>1050</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="211" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9543,10 +9543,10 @@
         <v>138</v>
       </c>
       <c r="F211" s="6" t="s">
-        <v>1051</v>
+        <v>1049</v>
       </c>
       <c r="G211" s="8" t="s">
-        <v>1052</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="212" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9566,10 +9566,10 @@
         <v>138</v>
       </c>
       <c r="F212" s="6" t="s">
-        <v>1053</v>
+        <v>1051</v>
       </c>
       <c r="G212" s="8" t="s">
-        <v>1054</v>
+        <v>1052</v>
       </c>
     </row>
     <row r="213" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9589,10 +9589,10 @@
         <v>138</v>
       </c>
       <c r="F213" s="6" t="s">
-        <v>1055</v>
+        <v>1053</v>
       </c>
       <c r="G213" s="8" t="s">
-        <v>1056</v>
+        <v>1054</v>
       </c>
     </row>
     <row r="214" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9612,10 +9612,10 @@
         <v>138</v>
       </c>
       <c r="F214" s="6" t="s">
-        <v>1057</v>
+        <v>1055</v>
       </c>
       <c r="G214" s="8" t="s">
-        <v>1058</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="215" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9635,10 +9635,10 @@
         <v>138</v>
       </c>
       <c r="F215" s="6" t="s">
-        <v>1059</v>
+        <v>1057</v>
       </c>
       <c r="G215" s="8" t="s">
-        <v>1060</v>
+        <v>1058</v>
       </c>
     </row>
     <row r="216" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9658,10 +9658,10 @@
         <v>138</v>
       </c>
       <c r="F216" s="6" t="s">
-        <v>1061</v>
+        <v>1059</v>
       </c>
       <c r="G216" s="8" t="s">
-        <v>1062</v>
+        <v>1060</v>
       </c>
     </row>
     <row r="217" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9681,10 +9681,10 @@
         <v>138</v>
       </c>
       <c r="F217" s="6" t="s">
-        <v>1063</v>
+        <v>1061</v>
       </c>
       <c r="G217" s="8" t="s">
-        <v>1064</v>
+        <v>1062</v>
       </c>
     </row>
     <row r="218" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -9704,10 +9704,10 @@
         <v>138</v>
       </c>
       <c r="F218" s="6" t="s">
-        <v>1065</v>
+        <v>1063</v>
       </c>
       <c r="G218" s="8" t="s">
-        <v>1066</v>
+        <v>1064</v>
       </c>
     </row>
     <row r="219" spans="1:7" x14ac:dyDescent="0.3">
@@ -9727,10 +9727,10 @@
         <v>138</v>
       </c>
       <c r="F219" s="9" t="s">
-        <v>1067</v>
+        <v>1065</v>
       </c>
       <c r="G219" s="10" t="s">
-        <v>1068</v>
+        <v>1066</v>
       </c>
     </row>
     <row r="220" spans="1:7" x14ac:dyDescent="0.3">
@@ -9750,10 +9750,10 @@
         <v>138</v>
       </c>
       <c r="F220" s="11" t="s">
-        <v>1069</v>
+        <v>1067</v>
       </c>
       <c r="G220" s="11" t="s">
-        <v>1070</v>
+        <v>1068</v>
       </c>
     </row>
     <row r="221" spans="1:7" x14ac:dyDescent="0.3">
@@ -9773,10 +9773,10 @@
         <v>138</v>
       </c>
       <c r="F221" s="11" t="s">
-        <v>1071</v>
+        <v>1069</v>
       </c>
       <c r="G221" s="11" t="s">
-        <v>1072</v>
+        <v>1070</v>
       </c>
     </row>
     <row r="222" spans="1:7" x14ac:dyDescent="0.3">
@@ -9796,10 +9796,10 @@
         <v>138</v>
       </c>
       <c r="F222" s="11" t="s">
-        <v>1073</v>
+        <v>1071</v>
       </c>
       <c r="G222" s="11" t="s">
-        <v>1074</v>
+        <v>1072</v>
       </c>
     </row>
     <row r="223" spans="1:7" x14ac:dyDescent="0.3">
@@ -9819,10 +9819,10 @@
         <v>138</v>
       </c>
       <c r="F223" s="11" t="s">
-        <v>1075</v>
+        <v>1073</v>
       </c>
       <c r="G223" s="11" t="s">
-        <v>1076</v>
+        <v>1074</v>
       </c>
     </row>
     <row r="224" spans="1:7" x14ac:dyDescent="0.3">
@@ -9842,10 +9842,10 @@
         <v>138</v>
       </c>
       <c r="F224" s="11" t="s">
-        <v>1077</v>
+        <v>1075</v>
       </c>
       <c r="G224" s="11" t="s">
-        <v>1078</v>
+        <v>1076</v>
       </c>
     </row>
     <row r="225" spans="1:7" x14ac:dyDescent="0.3">
@@ -9865,10 +9865,10 @@
         <v>138</v>
       </c>
       <c r="F225" s="11" t="s">
-        <v>1079</v>
+        <v>1077</v>
       </c>
       <c r="G225" s="11" t="s">
-        <v>1080</v>
+        <v>1078</v>
       </c>
     </row>
     <row r="226" spans="1:7" x14ac:dyDescent="0.3">
@@ -9888,10 +9888,10 @@
         <v>138</v>
       </c>
       <c r="F226" s="11" t="s">
-        <v>1081</v>
+        <v>1079</v>
       </c>
       <c r="G226" s="11" t="s">
-        <v>1082</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="227" spans="1:7" x14ac:dyDescent="0.3">
@@ -9911,10 +9911,10 @@
         <v>138</v>
       </c>
       <c r="F227" s="11" t="s">
-        <v>1083</v>
+        <v>1081</v>
       </c>
       <c r="G227" s="11" t="s">
-        <v>1084</v>
+        <v>1082</v>
       </c>
     </row>
     <row r="228" spans="1:7" x14ac:dyDescent="0.3">
@@ -9934,10 +9934,10 @@
         <v>138</v>
       </c>
       <c r="F228" s="11" t="s">
-        <v>1085</v>
+        <v>1083</v>
       </c>
       <c r="G228" s="11" t="s">
-        <v>1086</v>
+        <v>1084</v>
       </c>
     </row>
     <row r="229" spans="1:7" x14ac:dyDescent="0.3">
@@ -9957,10 +9957,10 @@
         <v>138</v>
       </c>
       <c r="F229" s="11" t="s">
-        <v>1087</v>
+        <v>1085</v>
       </c>
       <c r="G229" s="11" t="s">
-        <v>1088</v>
+        <v>1086</v>
       </c>
     </row>
     <row r="230" spans="1:7" x14ac:dyDescent="0.3">
@@ -9980,10 +9980,10 @@
         <v>138</v>
       </c>
       <c r="F230" s="11" t="s">
-        <v>1089</v>
+        <v>1087</v>
       </c>
       <c r="G230" s="11" t="s">
-        <v>1090</v>
+        <v>1088</v>
       </c>
     </row>
     <row r="231" spans="1:7" x14ac:dyDescent="0.3">
@@ -10003,10 +10003,10 @@
         <v>138</v>
       </c>
       <c r="F231" s="11" t="s">
-        <v>1091</v>
+        <v>1089</v>
       </c>
       <c r="G231" s="11" t="s">
-        <v>1092</v>
+        <v>1090</v>
       </c>
     </row>
     <row r="232" spans="1:7" x14ac:dyDescent="0.3">
@@ -10026,10 +10026,10 @@
         <v>138</v>
       </c>
       <c r="F232" s="11" t="s">
-        <v>1093</v>
+        <v>1091</v>
       </c>
       <c r="G232" s="11" t="s">
-        <v>1094</v>
+        <v>1092</v>
       </c>
     </row>
     <row r="233" spans="1:7" x14ac:dyDescent="0.3">
@@ -10049,10 +10049,10 @@
         <v>138</v>
       </c>
       <c r="F233" s="11" t="s">
-        <v>1095</v>
+        <v>1093</v>
       </c>
       <c r="G233" s="11" t="s">
-        <v>1096</v>
+        <v>1094</v>
       </c>
     </row>
     <row r="234" spans="1:7" x14ac:dyDescent="0.3">
@@ -10072,10 +10072,10 @@
         <v>138</v>
       </c>
       <c r="F234" s="11" t="s">
-        <v>1097</v>
+        <v>1095</v>
       </c>
       <c r="G234" s="11" t="s">
-        <v>1098</v>
+        <v>1096</v>
       </c>
     </row>
     <row r="235" spans="1:7" x14ac:dyDescent="0.3">
@@ -10095,10 +10095,10 @@
         <v>138</v>
       </c>
       <c r="F235" s="11" t="s">
-        <v>1099</v>
+        <v>1097</v>
       </c>
       <c r="G235" s="11" t="s">
-        <v>1100</v>
+        <v>1098</v>
       </c>
     </row>
     <row r="236" spans="1:7" x14ac:dyDescent="0.3">
@@ -10118,10 +10118,10 @@
         <v>138</v>
       </c>
       <c r="F236" s="11" t="s">
-        <v>1101</v>
+        <v>1099</v>
       </c>
       <c r="G236" s="11" t="s">
-        <v>1102</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="237" spans="1:7" x14ac:dyDescent="0.3">
@@ -10141,10 +10141,10 @@
         <v>138</v>
       </c>
       <c r="F237" s="11" t="s">
-        <v>1103</v>
+        <v>1101</v>
       </c>
       <c r="G237" s="11" t="s">
-        <v>1104</v>
+        <v>1102</v>
       </c>
     </row>
     <row r="238" spans="1:7" x14ac:dyDescent="0.3">
@@ -10164,10 +10164,10 @@
         <v>138</v>
       </c>
       <c r="F238" s="11" t="s">
-        <v>1105</v>
+        <v>1103</v>
       </c>
       <c r="G238" s="11" t="s">
-        <v>1106</v>
+        <v>1104</v>
       </c>
     </row>
     <row r="239" spans="1:7" x14ac:dyDescent="0.3">
@@ -10187,10 +10187,10 @@
         <v>138</v>
       </c>
       <c r="F239" s="11" t="s">
-        <v>1107</v>
+        <v>1105</v>
       </c>
       <c r="G239" s="11" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
     </row>
     <row r="240" spans="1:7" x14ac:dyDescent="0.3">
@@ -10210,10 +10210,10 @@
         <v>138</v>
       </c>
       <c r="F240" s="11" t="s">
-        <v>1109</v>
+        <v>1107</v>
       </c>
       <c r="G240" s="11" t="s">
-        <v>1110</v>
+        <v>1108</v>
       </c>
     </row>
     <row r="241" spans="1:7" x14ac:dyDescent="0.3">
@@ -10233,10 +10233,10 @@
         <v>138</v>
       </c>
       <c r="F241" s="11" t="s">
-        <v>1111</v>
+        <v>1109</v>
       </c>
       <c r="G241" s="11" t="s">
-        <v>1112</v>
+        <v>1110</v>
       </c>
     </row>
     <row r="242" spans="1:7" x14ac:dyDescent="0.3">
@@ -10256,10 +10256,10 @@
         <v>138</v>
       </c>
       <c r="F242" s="11" t="s">
-        <v>1113</v>
+        <v>1111</v>
       </c>
       <c r="G242" s="11" t="s">
-        <v>1114</v>
+        <v>1112</v>
       </c>
     </row>
     <row r="243" spans="1:7" x14ac:dyDescent="0.3">
@@ -10279,10 +10279,10 @@
         <v>138</v>
       </c>
       <c r="F243" s="11" t="s">
-        <v>1115</v>
+        <v>1113</v>
       </c>
       <c r="G243" s="11" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
     </row>
     <row r="244" spans="1:7" x14ac:dyDescent="0.3">
@@ -10302,10 +10302,10 @@
         <v>138</v>
       </c>
       <c r="F244" s="11" t="s">
-        <v>1117</v>
+        <v>1115</v>
       </c>
       <c r="G244" s="11" t="s">
-        <v>1118</v>
+        <v>1116</v>
       </c>
     </row>
     <row r="245" spans="1:7" x14ac:dyDescent="0.3">
@@ -10325,10 +10325,10 @@
         <v>138</v>
       </c>
       <c r="F245" s="11" t="s">
-        <v>1119</v>
+        <v>1117</v>
       </c>
       <c r="G245" s="11" t="s">
-        <v>1120</v>
+        <v>1118</v>
       </c>
     </row>
     <row r="246" spans="1:7" x14ac:dyDescent="0.3">
@@ -10348,10 +10348,10 @@
         <v>138</v>
       </c>
       <c r="F246" s="11" t="s">
-        <v>1121</v>
+        <v>1119</v>
       </c>
       <c r="G246" s="11" t="s">
-        <v>1122</v>
+        <v>1120</v>
       </c>
     </row>
     <row r="247" spans="1:7" x14ac:dyDescent="0.3">
@@ -10371,10 +10371,10 @@
         <v>138</v>
       </c>
       <c r="F247" s="11" t="s">
-        <v>1123</v>
+        <v>1121</v>
       </c>
       <c r="G247" s="11" t="s">
-        <v>1124</v>
+        <v>1122</v>
       </c>
     </row>
     <row r="248" spans="1:7" x14ac:dyDescent="0.3">
@@ -10394,10 +10394,10 @@
         <v>138</v>
       </c>
       <c r="F248" s="11" t="s">
-        <v>1125</v>
+        <v>1123</v>
       </c>
       <c r="G248" s="11" t="s">
-        <v>1126</v>
+        <v>1124</v>
       </c>
     </row>
     <row r="249" spans="1:7" x14ac:dyDescent="0.3">
@@ -10417,10 +10417,10 @@
         <v>138</v>
       </c>
       <c r="F249" s="11" t="s">
-        <v>1127</v>
+        <v>1125</v>
       </c>
       <c r="G249" s="11" t="s">
-        <v>1128</v>
+        <v>1126</v>
       </c>
     </row>
     <row r="250" spans="1:7" x14ac:dyDescent="0.3">
@@ -10440,10 +10440,10 @@
         <v>138</v>
       </c>
       <c r="F250" s="11" t="s">
-        <v>1129</v>
+        <v>1127</v>
       </c>
       <c r="G250" s="11" t="s">
-        <v>1130</v>
+        <v>1128</v>
       </c>
     </row>
     <row r="251" spans="1:7" x14ac:dyDescent="0.3">
@@ -10463,10 +10463,10 @@
         <v>138</v>
       </c>
       <c r="F251" s="11" t="s">
-        <v>1131</v>
+        <v>1129</v>
       </c>
       <c r="G251" s="11" t="s">
-        <v>1132</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="252" spans="1:7" x14ac:dyDescent="0.3">
@@ -10486,10 +10486,10 @@
         <v>138</v>
       </c>
       <c r="F252" s="11" t="s">
-        <v>1133</v>
+        <v>1131</v>
       </c>
       <c r="G252" s="11" t="s">
-        <v>1134</v>
+        <v>1132</v>
       </c>
     </row>
     <row r="253" spans="1:7" x14ac:dyDescent="0.3">
@@ -10509,10 +10509,10 @@
         <v>138</v>
       </c>
       <c r="F253" s="11" t="s">
-        <v>1135</v>
+        <v>1133</v>
       </c>
       <c r="G253" s="11" t="s">
-        <v>1136</v>
+        <v>1134</v>
       </c>
     </row>
     <row r="254" spans="1:7" x14ac:dyDescent="0.3">
@@ -10532,10 +10532,10 @@
         <v>138</v>
       </c>
       <c r="F254" s="11" t="s">
-        <v>1137</v>
+        <v>1135</v>
       </c>
       <c r="G254" s="11" t="s">
-        <v>1138</v>
+        <v>1136</v>
       </c>
     </row>
     <row r="255" spans="1:7" x14ac:dyDescent="0.3">
@@ -10555,10 +10555,10 @@
         <v>138</v>
       </c>
       <c r="F255" s="11" t="s">
-        <v>1139</v>
+        <v>1137</v>
       </c>
       <c r="G255" s="11" t="s">
-        <v>1140</v>
+        <v>1138</v>
       </c>
     </row>
     <row r="256" spans="1:7" x14ac:dyDescent="0.3">
@@ -10578,10 +10578,10 @@
         <v>138</v>
       </c>
       <c r="F256" s="11" t="s">
-        <v>1141</v>
+        <v>1139</v>
       </c>
       <c r="G256" s="11" t="s">
-        <v>1142</v>
+        <v>1140</v>
       </c>
     </row>
     <row r="257" spans="1:7" x14ac:dyDescent="0.3">
@@ -10601,10 +10601,10 @@
         <v>138</v>
       </c>
       <c r="F257" s="11" t="s">
-        <v>1143</v>
+        <v>1141</v>
       </c>
       <c r="G257" s="11" t="s">
-        <v>1144</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="258" spans="1:7" x14ac:dyDescent="0.3">
@@ -10624,10 +10624,10 @@
         <v>138</v>
       </c>
       <c r="F258" s="11" t="s">
-        <v>1145</v>
+        <v>1143</v>
       </c>
       <c r="G258" s="11" t="s">
-        <v>1146</v>
+        <v>1144</v>
       </c>
     </row>
     <row r="259" spans="1:7" x14ac:dyDescent="0.3">
@@ -10647,10 +10647,10 @@
         <v>138</v>
       </c>
       <c r="F259" s="11" t="s">
-        <v>1147</v>
+        <v>1145</v>
       </c>
       <c r="G259" s="11" t="s">
-        <v>1148</v>
+        <v>1146</v>
       </c>
     </row>
     <row r="260" spans="1:7" x14ac:dyDescent="0.3">
@@ -10670,10 +10670,10 @@
         <v>138</v>
       </c>
       <c r="F260" s="11" t="s">
-        <v>1149</v>
+        <v>1147</v>
       </c>
       <c r="G260" s="11" t="s">
-        <v>1150</v>
+        <v>1148</v>
       </c>
     </row>
     <row r="261" spans="1:7" x14ac:dyDescent="0.3">
@@ -10693,10 +10693,10 @@
         <v>138</v>
       </c>
       <c r="F261" s="11" t="s">
-        <v>1151</v>
+        <v>1149</v>
       </c>
       <c r="G261" s="11" t="s">
-        <v>1152</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="262" spans="1:7" x14ac:dyDescent="0.3">
@@ -10716,10 +10716,10 @@
         <v>138</v>
       </c>
       <c r="F262" s="11" t="s">
-        <v>1153</v>
+        <v>1151</v>
       </c>
       <c r="G262" s="11" t="s">
-        <v>1154</v>
+        <v>1152</v>
       </c>
     </row>
     <row r="263" spans="1:7" x14ac:dyDescent="0.3">
@@ -10739,10 +10739,10 @@
         <v>138</v>
       </c>
       <c r="F263" s="11" t="s">
-        <v>1155</v>
+        <v>1153</v>
       </c>
       <c r="G263" s="11" t="s">
-        <v>1156</v>
+        <v>1154</v>
       </c>
     </row>
     <row r="264" spans="1:7" x14ac:dyDescent="0.3">
@@ -10762,10 +10762,10 @@
         <v>138</v>
       </c>
       <c r="F264" s="11" t="s">
-        <v>1157</v>
+        <v>1155</v>
       </c>
       <c r="G264" s="11" t="s">
-        <v>1158</v>
+        <v>1156</v>
       </c>
     </row>
     <row r="265" spans="1:7" x14ac:dyDescent="0.3">
@@ -10785,10 +10785,10 @@
         <v>138</v>
       </c>
       <c r="F265" s="11" t="s">
-        <v>1159</v>
+        <v>1157</v>
       </c>
       <c r="G265" s="11" t="s">
-        <v>1160</v>
+        <v>1158</v>
       </c>
     </row>
     <row r="266" spans="1:7" x14ac:dyDescent="0.3">
@@ -10808,10 +10808,10 @@
         <v>138</v>
       </c>
       <c r="F266" s="11" t="s">
-        <v>1161</v>
+        <v>1159</v>
       </c>
       <c r="G266" s="11" t="s">
-        <v>1162</v>
+        <v>1160</v>
       </c>
     </row>
     <row r="267" spans="1:7" x14ac:dyDescent="0.3">
@@ -10831,10 +10831,10 @@
         <v>138</v>
       </c>
       <c r="F267" s="11" t="s">
-        <v>1163</v>
+        <v>1161</v>
       </c>
       <c r="G267" s="11" t="s">
-        <v>1164</v>
+        <v>1162</v>
       </c>
     </row>
     <row r="268" spans="1:7" x14ac:dyDescent="0.3">
@@ -10854,10 +10854,10 @@
         <v>138</v>
       </c>
       <c r="F268" s="11" t="s">
-        <v>1165</v>
+        <v>1163</v>
       </c>
       <c r="G268" s="11" t="s">
-        <v>1166</v>
+        <v>1164</v>
       </c>
     </row>
     <row r="269" spans="1:7" x14ac:dyDescent="0.3">
@@ -10877,10 +10877,10 @@
         <v>138</v>
       </c>
       <c r="F269" s="11" t="s">
-        <v>1167</v>
+        <v>1165</v>
       </c>
       <c r="G269" s="11" t="s">
-        <v>1168</v>
+        <v>1166</v>
       </c>
     </row>
     <row r="270" spans="1:7" x14ac:dyDescent="0.3">
@@ -10900,10 +10900,10 @@
         <v>138</v>
       </c>
       <c r="F270" s="11" t="s">
-        <v>1169</v>
+        <v>1167</v>
       </c>
       <c r="G270" s="11" t="s">
-        <v>1170</v>
+        <v>1168</v>
       </c>
     </row>
     <row r="271" spans="1:7" x14ac:dyDescent="0.3">
@@ -10923,10 +10923,10 @@
         <v>138</v>
       </c>
       <c r="F271" s="11" t="s">
-        <v>1171</v>
+        <v>1169</v>
       </c>
       <c r="G271" s="11" t="s">
-        <v>1172</v>
+        <v>1170</v>
       </c>
     </row>
     <row r="272" spans="1:7" x14ac:dyDescent="0.3">
@@ -10946,10 +10946,10 @@
         <v>138</v>
       </c>
       <c r="F272" s="11" t="s">
-        <v>1173</v>
+        <v>1171</v>
       </c>
       <c r="G272" s="11" t="s">
-        <v>1174</v>
+        <v>1172</v>
       </c>
     </row>
     <row r="273" spans="1:7" x14ac:dyDescent="0.3">
@@ -10969,10 +10969,10 @@
         <v>138</v>
       </c>
       <c r="F273" s="11" t="s">
-        <v>1175</v>
+        <v>1173</v>
       </c>
       <c r="G273" s="11" t="s">
-        <v>1176</v>
+        <v>1174</v>
       </c>
     </row>
     <row r="274" spans="1:7" x14ac:dyDescent="0.3">
@@ -10992,10 +10992,10 @@
         <v>138</v>
       </c>
       <c r="F274" s="11" t="s">
-        <v>1177</v>
+        <v>1175</v>
       </c>
       <c r="G274" s="11" t="s">
-        <v>1178</v>
+        <v>1176</v>
       </c>
     </row>
     <row r="275" spans="1:7" x14ac:dyDescent="0.3">
@@ -11015,10 +11015,10 @@
         <v>138</v>
       </c>
       <c r="F275" s="11" t="s">
-        <v>1179</v>
+        <v>1177</v>
       </c>
       <c r="G275" s="11" t="s">
-        <v>1180</v>
+        <v>1178</v>
       </c>
     </row>
     <row r="276" spans="1:7" x14ac:dyDescent="0.3">
@@ -11038,10 +11038,10 @@
         <v>138</v>
       </c>
       <c r="F276" s="11" t="s">
-        <v>1181</v>
+        <v>1179</v>
       </c>
       <c r="G276" s="11" t="s">
-        <v>1182</v>
+        <v>1180</v>
       </c>
     </row>
     <row r="277" spans="1:7" x14ac:dyDescent="0.3">
@@ -11061,10 +11061,10 @@
         <v>138</v>
       </c>
       <c r="F277" s="11" t="s">
-        <v>1183</v>
+        <v>1181</v>
       </c>
       <c r="G277" s="11" t="s">
-        <v>1184</v>
+        <v>1182</v>
       </c>
     </row>
     <row r="278" spans="1:7" x14ac:dyDescent="0.3">
@@ -11084,10 +11084,10 @@
         <v>138</v>
       </c>
       <c r="F278" s="11" t="s">
-        <v>1185</v>
+        <v>1183</v>
       </c>
       <c r="G278" s="11" t="s">
-        <v>1186</v>
+        <v>1184</v>
       </c>
     </row>
     <row r="279" spans="1:7" x14ac:dyDescent="0.3">
@@ -11107,10 +11107,10 @@
         <v>138</v>
       </c>
       <c r="F279" s="11" t="s">
-        <v>1187</v>
+        <v>1185</v>
       </c>
       <c r="G279" s="11" t="s">
-        <v>1188</v>
+        <v>1186</v>
       </c>
     </row>
     <row r="280" spans="1:7" x14ac:dyDescent="0.3">
@@ -11130,10 +11130,10 @@
         <v>138</v>
       </c>
       <c r="F280" s="11" t="s">
-        <v>1189</v>
+        <v>1187</v>
       </c>
       <c r="G280" s="11" t="s">
-        <v>1190</v>
+        <v>1188</v>
       </c>
     </row>
     <row r="281" spans="1:7" x14ac:dyDescent="0.3">
@@ -11153,10 +11153,10 @@
         <v>138</v>
       </c>
       <c r="F281" s="11" t="s">
-        <v>1191</v>
+        <v>1189</v>
       </c>
       <c r="G281" s="11" t="s">
-        <v>1192</v>
+        <v>1190</v>
       </c>
     </row>
     <row r="282" spans="1:7" x14ac:dyDescent="0.3">
@@ -11176,10 +11176,10 @@
         <v>601</v>
       </c>
       <c r="F282" s="11" t="s">
-        <v>1193</v>
+        <v>1191</v>
       </c>
       <c r="G282" s="11" t="s">
-        <v>1194</v>
+        <v>1192</v>
       </c>
     </row>
     <row r="283" spans="1:7" x14ac:dyDescent="0.3">
@@ -11199,10 +11199,10 @@
         <v>601</v>
       </c>
       <c r="F283" s="11" t="s">
-        <v>1195</v>
+        <v>1193</v>
       </c>
       <c r="G283" s="11" t="s">
-        <v>1196</v>
+        <v>1194</v>
       </c>
     </row>
     <row r="284" spans="1:7" x14ac:dyDescent="0.3">
@@ -11222,10 +11222,10 @@
         <v>601</v>
       </c>
       <c r="F284" s="11" t="s">
-        <v>1197</v>
+        <v>1195</v>
       </c>
       <c r="G284" s="11" t="s">
-        <v>1198</v>
+        <v>1196</v>
       </c>
     </row>
     <row r="285" spans="1:7" x14ac:dyDescent="0.3">
@@ -11245,10 +11245,10 @@
         <v>601</v>
       </c>
       <c r="F285" s="11" t="s">
-        <v>1199</v>
+        <v>1197</v>
       </c>
       <c r="G285" s="11" t="s">
-        <v>1200</v>
+        <v>1198</v>
       </c>
     </row>
     <row r="286" spans="1:7" x14ac:dyDescent="0.3">
@@ -11268,10 +11268,10 @@
         <v>601</v>
       </c>
       <c r="F286" s="11" t="s">
-        <v>1201</v>
+        <v>1199</v>
       </c>
       <c r="G286" s="11" t="s">
-        <v>1202</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="287" spans="1:7" x14ac:dyDescent="0.3">
@@ -11291,10 +11291,10 @@
         <v>601</v>
       </c>
       <c r="F287" s="11" t="s">
-        <v>1203</v>
+        <v>1201</v>
       </c>
       <c r="G287" s="11" t="s">
-        <v>1204</v>
+        <v>1202</v>
       </c>
     </row>
     <row r="288" spans="1:7" x14ac:dyDescent="0.3">
@@ -11314,10 +11314,10 @@
         <v>601</v>
       </c>
       <c r="F288" s="11" t="s">
-        <v>1205</v>
+        <v>1203</v>
       </c>
       <c r="G288" s="11" t="s">
-        <v>1206</v>
+        <v>1204</v>
       </c>
     </row>
     <row r="289" spans="1:7" x14ac:dyDescent="0.3">
@@ -11337,10 +11337,10 @@
         <v>601</v>
       </c>
       <c r="F289" s="11" t="s">
-        <v>1207</v>
+        <v>1205</v>
       </c>
       <c r="G289" s="11" t="s">
-        <v>1208</v>
+        <v>1206</v>
       </c>
     </row>
     <row r="290" spans="1:7" x14ac:dyDescent="0.3">
@@ -11360,10 +11360,10 @@
         <v>601</v>
       </c>
       <c r="F290" s="11" t="s">
-        <v>1209</v>
+        <v>1207</v>
       </c>
       <c r="G290" s="11" t="s">
-        <v>1210</v>
+        <v>1208</v>
       </c>
     </row>
     <row r="291" spans="1:7" x14ac:dyDescent="0.3">
@@ -11383,10 +11383,10 @@
         <v>601</v>
       </c>
       <c r="F291" s="11" t="s">
-        <v>1211</v>
+        <v>1209</v>
       </c>
       <c r="G291" s="11" t="s">
-        <v>1212</v>
+        <v>1210</v>
       </c>
     </row>
     <row r="292" spans="1:7" x14ac:dyDescent="0.3">
@@ -11406,10 +11406,10 @@
         <v>601</v>
       </c>
       <c r="F292" s="11" t="s">
-        <v>1213</v>
+        <v>1211</v>
       </c>
       <c r="G292" s="11" t="s">
-        <v>1214</v>
+        <v>1212</v>
       </c>
     </row>
     <row r="293" spans="1:7" x14ac:dyDescent="0.3">
@@ -11429,10 +11429,10 @@
         <v>601</v>
       </c>
       <c r="F293" s="11" t="s">
-        <v>1215</v>
+        <v>1213</v>
       </c>
       <c r="G293" s="11" t="s">
-        <v>1216</v>
+        <v>1214</v>
       </c>
     </row>
     <row r="294" spans="1:7" x14ac:dyDescent="0.3">
@@ -11452,10 +11452,10 @@
         <v>601</v>
       </c>
       <c r="F294" s="11" t="s">
-        <v>1217</v>
+        <v>1215</v>
       </c>
       <c r="G294" s="11" t="s">
-        <v>1218</v>
+        <v>1216</v>
       </c>
     </row>
     <row r="295" spans="1:7" x14ac:dyDescent="0.3">
@@ -11475,10 +11475,10 @@
         <v>601</v>
       </c>
       <c r="F295" s="11" t="s">
-        <v>1219</v>
+        <v>1217</v>
       </c>
       <c r="G295" s="11" t="s">
-        <v>1220</v>
+        <v>1218</v>
       </c>
     </row>
     <row r="296" spans="1:7" x14ac:dyDescent="0.3">
@@ -11498,10 +11498,10 @@
         <v>601</v>
       </c>
       <c r="F296" s="11" t="s">
-        <v>1221</v>
+        <v>1219</v>
       </c>
       <c r="G296" s="11" t="s">
-        <v>1222</v>
+        <v>1220</v>
       </c>
     </row>
     <row r="297" spans="1:7" x14ac:dyDescent="0.3">
@@ -11521,10 +11521,10 @@
         <v>601</v>
       </c>
       <c r="F297" s="11" t="s">
-        <v>1223</v>
+        <v>1221</v>
       </c>
       <c r="G297" s="11" t="s">
-        <v>1224</v>
+        <v>1222</v>
       </c>
     </row>
     <row r="298" spans="1:7" x14ac:dyDescent="0.3">
@@ -11544,10 +11544,10 @@
         <v>138</v>
       </c>
       <c r="F298" s="11" t="s">
-        <v>1225</v>
+        <v>1223</v>
       </c>
       <c r="G298" s="11" t="s">
-        <v>1226</v>
+        <v>1224</v>
       </c>
     </row>
     <row r="299" spans="1:7" x14ac:dyDescent="0.3">
@@ -11567,10 +11567,10 @@
         <v>138</v>
       </c>
       <c r="F299" s="11" t="s">
-        <v>1227</v>
+        <v>1225</v>
       </c>
       <c r="G299" s="11" t="s">
-        <v>1228</v>
+        <v>1226</v>
       </c>
     </row>
     <row r="300" spans="1:7" x14ac:dyDescent="0.3">
@@ -11590,10 +11590,10 @@
         <v>138</v>
       </c>
       <c r="F300" s="11" t="s">
-        <v>1229</v>
+        <v>1227</v>
       </c>
       <c r="G300" s="11" t="s">
-        <v>1230</v>
+        <v>1228</v>
       </c>
     </row>
     <row r="301" spans="1:7" x14ac:dyDescent="0.3">
@@ -11613,10 +11613,10 @@
         <v>138</v>
       </c>
       <c r="F301" s="11" t="s">
-        <v>1231</v>
+        <v>1229</v>
       </c>
       <c r="G301" s="11" t="s">
-        <v>1232</v>
+        <v>1230</v>
       </c>
     </row>
     <row r="302" spans="1:7" x14ac:dyDescent="0.3">
@@ -11636,10 +11636,10 @@
         <v>138</v>
       </c>
       <c r="F302" s="11" t="s">
-        <v>1233</v>
+        <v>1231</v>
       </c>
       <c r="G302" s="11" t="s">
-        <v>1234</v>
+        <v>1232</v>
       </c>
     </row>
     <row r="303" spans="1:7" x14ac:dyDescent="0.3">
@@ -11659,10 +11659,10 @@
         <v>138</v>
       </c>
       <c r="F303" s="11" t="s">
-        <v>1235</v>
+        <v>1233</v>
       </c>
       <c r="G303" s="11" t="s">
-        <v>1236</v>
+        <v>1234</v>
       </c>
     </row>
     <row r="304" spans="1:7" x14ac:dyDescent="0.3">
@@ -11682,10 +11682,10 @@
         <v>138</v>
       </c>
       <c r="F304" s="11" t="s">
-        <v>1237</v>
+        <v>1235</v>
       </c>
       <c r="G304" s="11" t="s">
-        <v>1238</v>
+        <v>1236</v>
       </c>
     </row>
     <row r="305" spans="1:7" x14ac:dyDescent="0.3">
@@ -11705,10 +11705,10 @@
         <v>138</v>
       </c>
       <c r="F305" s="11" t="s">
-        <v>1239</v>
+        <v>1237</v>
       </c>
       <c r="G305" s="11" t="s">
-        <v>1240</v>
+        <v>1238</v>
       </c>
     </row>
     <row r="306" spans="1:7" x14ac:dyDescent="0.3">
@@ -11728,10 +11728,10 @@
         <v>138</v>
       </c>
       <c r="F306" s="11" t="s">
-        <v>1241</v>
+        <v>1239</v>
       </c>
       <c r="G306" s="11" t="s">
-        <v>1242</v>
+        <v>1240</v>
       </c>
     </row>
     <row r="307" spans="1:7" x14ac:dyDescent="0.3">
@@ -11751,10 +11751,10 @@
         <v>138</v>
       </c>
       <c r="F307" s="11" t="s">
-        <v>1243</v>
+        <v>1241</v>
       </c>
       <c r="G307" s="11" t="s">
-        <v>1244</v>
+        <v>1242</v>
       </c>
     </row>
     <row r="308" spans="1:7" x14ac:dyDescent="0.3">
@@ -11774,10 +11774,10 @@
         <v>601</v>
       </c>
       <c r="F308" s="11" t="s">
-        <v>1245</v>
+        <v>1243</v>
       </c>
       <c r="G308" s="11" t="s">
-        <v>1246</v>
+        <v>1244</v>
       </c>
     </row>
     <row r="309" spans="1:7" x14ac:dyDescent="0.3">
@@ -11797,10 +11797,10 @@
         <v>601</v>
       </c>
       <c r="F309" s="11" t="s">
-        <v>1247</v>
+        <v>1245</v>
       </c>
       <c r="G309" s="11" t="s">
-        <v>1248</v>
+        <v>1246</v>
       </c>
     </row>
     <row r="310" spans="1:7" x14ac:dyDescent="0.3">
@@ -11820,10 +11820,10 @@
         <v>601</v>
       </c>
       <c r="F310" s="11" t="s">
-        <v>1249</v>
+        <v>1247</v>
       </c>
       <c r="G310" s="11" t="s">
-        <v>1250</v>
+        <v>1248</v>
       </c>
     </row>
     <row r="311" spans="1:7" x14ac:dyDescent="0.3">
@@ -11843,10 +11843,10 @@
         <v>601</v>
       </c>
       <c r="F311" s="11" t="s">
-        <v>1251</v>
+        <v>1249</v>
       </c>
       <c r="G311" s="11" t="s">
-        <v>1252</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="312" spans="1:7" x14ac:dyDescent="0.3">
@@ -11866,10 +11866,10 @@
         <v>601</v>
       </c>
       <c r="F312" s="11" t="s">
-        <v>1253</v>
+        <v>1251</v>
       </c>
       <c r="G312" s="11" t="s">
-        <v>1254</v>
+        <v>1252</v>
       </c>
     </row>
     <row r="313" spans="1:7" x14ac:dyDescent="0.3">
@@ -11889,10 +11889,10 @@
         <v>601</v>
       </c>
       <c r="F313" s="11" t="s">
-        <v>1255</v>
+        <v>1253</v>
       </c>
       <c r="G313" s="11" t="s">
-        <v>1256</v>
+        <v>1254</v>
       </c>
     </row>
     <row r="314" spans="1:7" x14ac:dyDescent="0.3">
@@ -11912,10 +11912,10 @@
         <v>601</v>
       </c>
       <c r="F314" s="11" t="s">
-        <v>1257</v>
+        <v>1255</v>
       </c>
       <c r="G314" s="11" t="s">
-        <v>1258</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="315" spans="1:7" x14ac:dyDescent="0.3">
@@ -11935,10 +11935,10 @@
         <v>601</v>
       </c>
       <c r="F315" s="11" t="s">
-        <v>1259</v>
+        <v>1257</v>
       </c>
       <c r="G315" s="11" t="s">
-        <v>1260</v>
+        <v>1258</v>
       </c>
     </row>
     <row r="316" spans="1:7" x14ac:dyDescent="0.3">
@@ -11958,10 +11958,10 @@
         <v>601</v>
       </c>
       <c r="F316" s="11" t="s">
-        <v>1261</v>
+        <v>1259</v>
       </c>
       <c r="G316" s="11" t="s">
-        <v>1262</v>
+        <v>1260</v>
       </c>
     </row>
     <row r="317" spans="1:7" x14ac:dyDescent="0.3">
@@ -11981,10 +11981,10 @@
         <v>601</v>
       </c>
       <c r="F317" s="11" t="s">
-        <v>1263</v>
+        <v>1261</v>
       </c>
       <c r="G317" s="11" t="s">
-        <v>1264</v>
+        <v>1262</v>
       </c>
     </row>
     <row r="318" spans="1:7" x14ac:dyDescent="0.3">
@@ -12004,10 +12004,10 @@
         <v>601</v>
       </c>
       <c r="F318" s="11" t="s">
-        <v>1265</v>
+        <v>1263</v>
       </c>
       <c r="G318" s="11" t="s">
-        <v>1266</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="319" spans="1:7" x14ac:dyDescent="0.3">
@@ -12027,10 +12027,10 @@
         <v>601</v>
       </c>
       <c r="F319" s="11" t="s">
-        <v>1267</v>
+        <v>1265</v>
       </c>
       <c r="G319" s="11" t="s">
-        <v>1268</v>
+        <v>1266</v>
       </c>
     </row>
     <row r="320" spans="1:7" x14ac:dyDescent="0.3">
@@ -12050,10 +12050,10 @@
         <v>601</v>
       </c>
       <c r="F320" s="11" t="s">
-        <v>1269</v>
+        <v>1267</v>
       </c>
       <c r="G320" s="11" t="s">
-        <v>1270</v>
+        <v>1268</v>
       </c>
     </row>
     <row r="321" spans="1:7" x14ac:dyDescent="0.3">
@@ -12073,10 +12073,10 @@
         <v>601</v>
       </c>
       <c r="F321" s="11" t="s">
-        <v>1271</v>
+        <v>1269</v>
       </c>
       <c r="G321" s="11" t="s">
-        <v>1272</v>
+        <v>1270</v>
       </c>
     </row>
     <row r="322" spans="1:7" x14ac:dyDescent="0.3">
@@ -12096,10 +12096,10 @@
         <v>601</v>
       </c>
       <c r="F322" s="11" t="s">
-        <v>1273</v>
+        <v>1271</v>
       </c>
       <c r="G322" s="11" t="s">
-        <v>1274</v>
+        <v>1272</v>
       </c>
     </row>
     <row r="323" spans="1:7" x14ac:dyDescent="0.3">
@@ -12119,10 +12119,10 @@
         <v>601</v>
       </c>
       <c r="F323" s="11" t="s">
-        <v>1275</v>
+        <v>1273</v>
       </c>
       <c r="G323" s="11" t="s">
-        <v>1276</v>
+        <v>1274</v>
       </c>
     </row>
     <row r="324" spans="1:7" x14ac:dyDescent="0.3">
@@ -12142,10 +12142,10 @@
         <v>601</v>
       </c>
       <c r="F324" s="11" t="s">
-        <v>1277</v>
+        <v>1275</v>
       </c>
       <c r="G324" s="11" t="s">
-        <v>1278</v>
+        <v>1276</v>
       </c>
     </row>
     <row r="325" spans="1:7" x14ac:dyDescent="0.3">
@@ -12165,10 +12165,10 @@
         <v>601</v>
       </c>
       <c r="F325" s="11" t="s">
-        <v>1279</v>
+        <v>1277</v>
       </c>
       <c r="G325" s="11" t="s">
-        <v>1280</v>
+        <v>1278</v>
       </c>
     </row>
     <row r="326" spans="1:7" x14ac:dyDescent="0.3">
@@ -12188,10 +12188,10 @@
         <v>601</v>
       </c>
       <c r="F326" s="11" t="s">
-        <v>1281</v>
+        <v>1279</v>
       </c>
       <c r="G326" s="11" t="s">
-        <v>1282</v>
+        <v>1280</v>
       </c>
     </row>
     <row r="327" spans="1:7" x14ac:dyDescent="0.3">
@@ -12211,10 +12211,10 @@
         <v>601</v>
       </c>
       <c r="F327" s="11" t="s">
-        <v>1283</v>
+        <v>1281</v>
       </c>
       <c r="G327" s="11" t="s">
-        <v>1284</v>
+        <v>1282</v>
       </c>
     </row>
     <row r="328" spans="1:7" x14ac:dyDescent="0.3">
@@ -12234,10 +12234,10 @@
         <v>601</v>
       </c>
       <c r="F328" s="11" t="s">
-        <v>1285</v>
+        <v>1283</v>
       </c>
       <c r="G328" s="11" t="s">
-        <v>1286</v>
+        <v>1284</v>
       </c>
     </row>
     <row r="329" spans="1:7" x14ac:dyDescent="0.3">
@@ -12257,10 +12257,10 @@
         <v>601</v>
       </c>
       <c r="F329" s="11" t="s">
-        <v>1287</v>
+        <v>1285</v>
       </c>
       <c r="G329" s="11" t="s">
-        <v>1288</v>
+        <v>1286</v>
       </c>
     </row>
     <row r="330" spans="1:7" x14ac:dyDescent="0.3">
@@ -12280,10 +12280,10 @@
         <v>601</v>
       </c>
       <c r="F330" s="11" t="s">
-        <v>1289</v>
+        <v>1287</v>
       </c>
       <c r="G330" s="11" t="s">
-        <v>1290</v>
+        <v>1288</v>
       </c>
     </row>
     <row r="331" spans="1:7" x14ac:dyDescent="0.3">
@@ -12303,10 +12303,10 @@
         <v>601</v>
       </c>
       <c r="F331" s="11" t="s">
-        <v>1291</v>
+        <v>1289</v>
       </c>
       <c r="G331" s="11" t="s">
-        <v>1292</v>
+        <v>1290</v>
       </c>
     </row>
     <row r="332" spans="1:7" x14ac:dyDescent="0.3">
@@ -12326,10 +12326,10 @@
         <v>601</v>
       </c>
       <c r="F332" s="11" t="s">
-        <v>1293</v>
+        <v>1291</v>
       </c>
       <c r="G332" s="11" t="s">
-        <v>1294</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="333" spans="1:7" x14ac:dyDescent="0.3">
@@ -12349,10 +12349,10 @@
         <v>601</v>
       </c>
       <c r="F333" s="11" t="s">
-        <v>1295</v>
+        <v>1293</v>
       </c>
       <c r="G333" s="11" t="s">
-        <v>1296</v>
+        <v>1294</v>
       </c>
     </row>
     <row r="334" spans="1:7" x14ac:dyDescent="0.3">
@@ -12372,10 +12372,10 @@
         <v>601</v>
       </c>
       <c r="F334" s="11" t="s">
-        <v>1297</v>
+        <v>1295</v>
       </c>
       <c r="G334" s="11" t="s">
-        <v>1298</v>
+        <v>1296</v>
       </c>
     </row>
     <row r="335" spans="1:7" x14ac:dyDescent="0.3">
@@ -12395,10 +12395,10 @@
         <v>601</v>
       </c>
       <c r="F335" s="11" t="s">
-        <v>1299</v>
+        <v>1297</v>
       </c>
       <c r="G335" s="11" t="s">
-        <v>1300</v>
+        <v>1298</v>
       </c>
     </row>
   </sheetData>

</xml_diff>